<commit_message>
Fix 37 verification findings: executable confirmation channels, null-watermark rule, Drive report versioning, A/B single-factor rule, letter compliance (signatures, gatekeeper, UTM, subjects), lock recovery, bounce accounting
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -612,7 +612,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>SPA для двоих — готовый сегмент для рекламы</t>
+          <t>SPA для двоих — недооценённый сегмент LAKSMI</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Ориентиры: reply rate 3–7% норма, &lt;2% после 50 писем — менять тему/оффер; ответы без созвонов — менять CTA; отписки &gt;10% — менять базу. Решения — только по дозревшим когортам (лист 3).</t>
+          <t>Ориентиры (источник — playbook.md, «Ориентиры метрик» и «Ворота выборки»): reply rate 3–7% норма, &lt;2% при ≥50 доставленных — тревога; bounce &gt;5% — тревога; тема/абзац — только по A/B ≥40 отправок на вариант; отказ от ниши — 0 ответов на 60 отправках или (bounce+отписки) &gt;15%; пересмотр базы — отписки+жалобы ≥8. Решения — только по дозревшим когортам ≥14 дней (лист 3) и через подтверждение Яны.</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Старт рассылки: 10 писем (бьюти 4, обучение 3, медицина 3), оффер — платный трафик + SMM, CTA — бесплатная консультация. Ожидание: reply rate ≥3%. Решения принимать после ~30–50 отправленных писем.</t>
+          <t>Старт рассылки: 10 писем подготовлено (бьюти 4, обучение 3, медицина 3), отправка ожидает подтверждения Яны. Блокер №1 — переавторизация Gmail (не видим ответы). С 07.07 запущен EXP-001-cta. Ожидание: reply rate ≥3% от доставленных; решения — после дозревания когорт (≥14 дней).</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2000,6 +2000,77 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>EXP-001-cta</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CTA с микро-ценностью («пришлю мини-разбор в 10 строк — ответьте „да“») даст больше ответов, чем прямой CTA на созвон, потому что порог согласия ниже</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CTA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>мини-разбор (ответьте «да»)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>созвон 20 минут (текущий)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>REDESIGN-v2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Полная переработка системы по итогам аудита (59 находок): подтверждение отправки, статусы v2, Asana-интеграция, A/B, когортная аналитика, надёжность запусков</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>sales-agent/*</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>применено</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>исчезнут потерянные лиды и невидимые ответы; появится измеримый цикл улучшения стратегии</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Batch 07.07: 10 deep-researched leads (social recon, LPR), first A/B batch EXP-001-cta, 3 backlog
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -20,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -66,13 +67,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -441,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S13"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -569,7 +571,9 @@
       <c r="B2" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Клиника эстетической медицины «Сибирская»</t>
@@ -617,7 +621,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N2" s="2" t="n"/>
@@ -639,7 +643,9 @@
       <c r="B3" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C3" s="2" t="n"/>
+      <c r="C3" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>КВК — Клиника врачебной косметологии</t>
@@ -687,7 +693,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N3" s="2" t="n"/>
@@ -709,7 +715,9 @@
       <c r="B4" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C4" s="2" t="n"/>
+      <c r="C4" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Студия маникюра LAKи</t>
@@ -757,7 +765,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N4" s="2" t="n"/>
@@ -779,7 +787,9 @@
       <c r="B5" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C5" s="2" t="n"/>
+      <c r="C5" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>SPA-салон LAKSMI</t>
@@ -827,7 +837,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N5" s="2" t="n"/>
@@ -849,7 +859,9 @@
       <c r="B6" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C6" s="2" t="n"/>
+      <c r="C6" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>Школа иностранных языков Star Talk</t>
@@ -897,7 +909,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N6" s="2" t="n"/>
@@ -919,7 +931,9 @@
       <c r="B7" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C7" s="2" t="n"/>
+      <c r="C7" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>Детская онлайн-школа программирования Hello World</t>
@@ -967,7 +981,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N7" s="2" t="n"/>
@@ -989,7 +1003,9 @@
       <c r="B8" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C8" s="2" t="n"/>
+      <c r="C8" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>Художественная школа «Арт-Идея»</t>
@@ -1037,7 +1053,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N8" s="2" t="n"/>
@@ -1059,7 +1075,9 @@
       <c r="B9" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C9" s="2" t="n"/>
+      <c r="C9" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Лика Клиник (косметология)</t>
@@ -1107,7 +1125,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N9" s="2" t="n"/>
@@ -1129,7 +1147,9 @@
       <c r="B10" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C10" s="2" t="n"/>
+      <c r="C10" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>Стоматология «Классик Дент»</t>
@@ -1177,7 +1197,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N10" s="2" t="n"/>
@@ -1199,7 +1219,9 @@
       <c r="B11" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C11" s="2" t="n"/>
+      <c r="C11" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Медицинский центр «Я здоров!»</t>
@@ -1247,7 +1269,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N11" s="2" t="n"/>
@@ -1399,6 +1421,916 @@
       <c r="S13" t="inlineStr">
         <is>
           <t>Резерв: семейная многопрофильная клиника, слабее персонализация — дособрать факты перед письмом</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Клиника эстетической медицины «Алтика»</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Смагин Алексей Владимирович (директор)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>info@altika-clinic.ru</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://altika-clinic.ru/</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Идея по записям для «Алтики»</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n"/>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="n"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>16 лет, ТОП-клиник Сибири 2023; широкая линейка (лазер, вес, подология, трихология); брендовый спрос уходит агрегаторам || Соцсети: VK указан в контактах, но не находится в поиске; 2ГИС 4.7 (302 оценки); негатив — про администраторов</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Клиника врачебной косметологии «Совершенство»</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Казань</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>info@sovershenstvo-clinic.ru</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://sovershenstvo-clinic.ru/</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Идея по записям для «Совершенства»</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="n"/>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2" t="n"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>С 2017, аппаратная база InMode; раздел «Акции» на сайте — готовые офферы без трафика; врачи Эльвира Асхатовна, Ляйля Рамиловна || Соцсети: VK/TG не находятся; ПроДокторов 29 положительных отзывов</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Terra del Sol (центр красоты)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Арзаманскина М. С. (гендиректор)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>terradel.sol@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://terraspa.ru/</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Идея по записям для Terra del Sol</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n"/>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="2" t="n"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>19+ лет, 2 филиала (Восход 14/1, пл. К. Маркса); запись только по телефону; устаревший сайт без трафика || Соцсети: VK vk.com/terradelsol; Фламп/2ГИС 4.5 (~130 отзывов), хвалят косметолога Элеонору Винник и стилиста Татьяну Евдокимову</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Салон красоты «Красивые Люди»</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Казань</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Виктор (директор, личный email на сайте)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>viktoroff2011@gmail.com</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>personal</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://xn----7sbb0bhbmbddc4a.xn--p1ai/</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Идея по записям для «Красивых Людей»</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="n"/>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="2" t="n"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Полный комплекс услуг; личный gmail директора — короткий цикл сделки; нет онлайн-записи || Соцсети: VK/IG-ссылки на сайте, активного сообщества нет; Zoon/Фламп: хвалят стилиста Мане (Air Touch), мастеров Светлану и Виктора</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Школа рисования «Найди Себя»</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>info@naydisebya.ru</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://naydisebya.ru</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Ученики для «Найди Себя» из ВКонтакте</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n"/>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="2" t="n"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Profieng — онлайн-школа английского</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>info@profieng.ru</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://profieng.ru</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Ученики к учебному году для Profieng</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n"/>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="2" t="n"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>IELTS/TOEFL/ЕГЭ + дети 4–12; сезонное окно — набор к учебному году; конкуренты (Skyeng) активно закупают трафик || Соцсети: VK/TG не видны в поиске; 20 отзывов на Kurshub (хвалят цену и расписание); Zoon, 2ГИС</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Школа шитья «Хочу Шить»</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Москва и Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Мария Амочаева (основатель)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>info@wanttosew.ru</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://wanttosew.ru</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Идея для «Хочу Шить» к осеннему набору</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n"/>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="2" t="n"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Огромная контентная база и лид-магниты (выкройки, вебинары) без платного трафика; офлайн Мск+СПб + онлайн — идеальный матч под кейс Кинезио || Соцсети: Личный бренд Марии в IG @mari_amochaeva (заблокирован); YouTube + Rutube 514 подборок; VK/TG школы не видны; блог на сайте заброшен (статья 2020 г.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Клиника медицинской косметологии «Ланцетъ»</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Нижний Новгород</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>info@lancette-nn.ru</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://lancette-nn.ru</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Пациентки для «Ланцета» — не только с ПроДокторов</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="n"/>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="2" t="n"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Премиум: БЦ Corner Place, врачи из моск. института пластической хирургии, чек до 56 200 ₽ — юнит-экономика Директа сходится с запасом || Соцсети: VK/TG/IG не находятся; ПроДокторов 170 отзывов, 18 врачей</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника «Визави»</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Евгений Леонидович (главный врач)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>vizavi-info@mail.ru</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://www.vizavi-ekb.ru</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Свои пациенты для «Визави» — без агрегаторов</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n"/>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="2" t="n"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>«Центр Стоматологии»</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Казань</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>centrstomat@mail.ru</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://www.xn--80aaakvedmgitccb3bqd3v.xn--p1ai/</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Прямые записи для «Центра Стоматологии»</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="n"/>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="2" t="n"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: Единственная соцстраница — заблокированный Facebook; Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Timeless (студия массажа и макияжа)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>info@timeless-studio.ru</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://timeless-studio.ru/</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n"/>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="2" t="n"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Резерв: рейтинг ниже конкурентов, нет ЛПР; anti-age авторские методики — фактура для креативов || Соцсети: IG @timeless_studio_massage основной канал; VK не найден; Zoon 3.4; 2 филиала</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Триарс — школа рисования</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Казань</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>info@triars.ru</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://triars.ru</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="n"/>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="2" t="n"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Стоматология «21 Век»</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Казань</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>stom.21@mail.ru</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://stomatologia21vek.ru</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n"/>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="2" t="n"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1</t>
         </is>
       </c>
     </row>
@@ -1413,7 +2345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1440,7 +2372,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -1470,7 +2402,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -1490,7 +2422,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -1509,6 +2441,9 @@
           <t>Reply rate (от доставленных)</t>
         </is>
       </c>
+      <c r="B10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1536,6 +2471,9 @@
           <t>Конверсия доставлено → созвон</t>
         </is>
       </c>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1611,54 +2549,85 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>По вариантам письма (A/B)</t>
-        </is>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>Сегмент</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>Отправлено</t>
-        </is>
-      </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>Bounce</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="inlineStr">
-        <is>
-          <t>Ответов</t>
-        </is>
-      </c>
-      <c r="E23" s="1" t="inlineStr">
-        <is>
-          <t>Reply rate</t>
-        </is>
-      </c>
-      <c r="F23" s="1" t="inlineStr">
-        <is>
-          <t>Созвонов</t>
-        </is>
-      </c>
-      <c r="G23" s="1" t="inlineStr">
-        <is>
-          <t>Конверсия</t>
-        </is>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>По типу ящика</t>
+          <t>По вариантам письма (A/B)</t>
         </is>
       </c>
     </row>
@@ -1699,52 +2668,196 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>10</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>По типу ящика</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Сегмент</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>Отправлено</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>Bounce</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>Ответов</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Reply rate</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>Созвонов</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>Конверсия</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>По наличию имени ЛПР</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>Сегмент</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>Отправлено</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C34" s="1" t="inlineStr">
         <is>
           <t>Bounce</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D34" s="1" t="inlineStr">
         <is>
           <t>Ответов</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E34" s="1" t="inlineStr">
         <is>
           <t>Reply rate</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>Созвонов</t>
         </is>
       </c>
-      <c r="G29" s="1" t="inlineStr">
+      <c r="G34" s="1" t="inlineStr">
         <is>
           <t>Конверсия</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>без имени</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>7</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>имя известно</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Ориентиры (источник — playbook.md, «Ориентиры метрик» и «Ворота выборки»): reply rate 3–7% норма, &lt;2% при ≥50 доставленных — тревога; bounce &gt;5% — тревога; тема/абзац — только по A/B ≥40 отправок на вариант; отказ от ниши — 0 ответов на 60 отправках или (bounce+отписки) &gt;15%; пересмотр базы — отписки+жалобы ≥8. Решения — только по дозревшим когортам ≥14 дней (лист 3) и через подтверждение Яны.</t>
         </is>
@@ -1761,7 +2874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1837,6 +2950,48 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Когорта дозрела?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>нет (&lt;14 дн)</t>
         </is>
       </c>
     </row>
@@ -1899,10 +3054,10 @@
         <v>46209</v>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1910,7 +3065,7 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Старт рассылки: 10 писем подготовлено (бьюти 4, обучение 3, медицина 3), отправка ожидает подтверждения Яны. Блокер №1 — переавторизация Gmail (не видим ответы). С 07.07 запущен EXP-001-cta. Ожидание: reply rate ≥3% от доставленных; решения — после дозревания когорт (≥14 дней).</t>
         </is>
@@ -1932,7 +3087,7 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="4" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rebuild 9 batch-2 drafts after social recon v2 (Yana caught false 'no VK' claim for Altika); replay Asana send-task; clear pending queue
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -1490,7 +1490,7 @@
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>16 лет, ТОП-клиник Сибири 2023; широкая линейка (лазер, вес, подология, трихология); брендовый спрос уходит агрегаторам || Соцсети: VK указан в контактах, но не находится в поиске; 2ГИС 4.7 (302 оценки); негатив — про администраторов</t>
+          <t>16 лет, ТОП-клиник Сибири 2023; широкая линейка (лазер, вес, подология, трихология); брендовый спрос уходит агрегаторам || Соцсети: VK указан в контактах, но не находится в поиске; 2ГИС 4.7 (302 оценки); негатив — про администраторов || СОЦРАЗВЕДКА v2 (07.07, после ошибки): ВК ЕСТЬ — vk.com/altikansk (подтверждено Яной; сайт заявляет ВК/WhatsApp/TG, страница ВК не индексируется поиском). Письмо пересобрано: зацепка на репутации+ВК, утверждение об отсутствии убрано</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>С 2017, аппаратная база InMode; раздел «Акции» на сайте — готовые офферы без трафика; врачи Эльвира Асхатовна, Ляйля Рамиловна || Соцсети: VK/TG не находятся; ПроДокторов 29 положительных отзывов</t>
+          <t>С 2017, аппаратная база InMode; раздел «Акции» на сайте — готовые офферы без трафика; врачи Эльвира Асхатовна, Ляйля Рамиловна || Соцсети: VK/TG не находятся; ПроДокторов 29 положительных отзывов || СОЦРАЗВЕДКА v2 (07.07): сайт заявляет ВК и Telegram (сниппеты контактов); IG @sovershenstvo_clinic. Письмо пересобрано: зацепка на разделе «Акции» без утверждений об отсутствии соцсетей</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Полный комплекс услуг; личный gmail директора — короткий цикл сделки; нет онлайн-записи || Соцсети: VK/IG-ссылки на сайте, активного сообщества нет; Zoon/Фламп: хвалят стилиста Мане (Air Touch), мастеров Светлану и Виктора</t>
+          <t>Полный комплекс услуг; личный gmail директора — короткий цикл сделки; нет онлайн-записи || Соцсети: VK/IG-ссылки на сайте, активного сообщества нет; Zoon/Фламп: хвалят стилиста Мане (Air Touch), мастеров Светлану и Виктора || СОЦРАЗВЕДКА v2 (07.07): yell.ru заявляет VK/IG; вероятный IG @krasivielyudi_official (принадлежность не подтверждена — тёзки в других городах). Письмо пересобрано: убрано «соцсети почти не живут», мягкая формулировка про карты/сарафан</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3</t>
+          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3 || СОЦРАЗВЕДКА v2 (07.07): Telegram-канал ЕСТЬ — t.me/naydisebyamsk; IG @naydisebya_ru 8,2K + @naydisebya.online; ВК не найден по сниппетам (не подтверждено). Письмо пересобрано: TG признан активом, утверждение «TG не развит» убрано</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>IELTS/TOEFL/ЕГЭ + дети 4–12; сезонное окно — набор к учебному году; конкуренты (Skyeng) активно закупают трафик || Соцсети: VK/TG не видны в поиске; 20 отзывов на Kurshub (хвалят цену и расписание); Zoon, 2ГИС</t>
+          <t>IELTS/TOEFL/ЕГЭ + дети 4–12; сезонное окно — набор к учебному году; конкуренты (Skyeng) активно закупают трафик || Соцсети: VK/TG не видны в поиске; 20 отзывов на Kurshub (хвалят цену и расписание); Zoon, 2ГИС || СОЦРАЗВЕДКА v2 (07.07): сайт на странице контактов заявляет YouTube и ВКонтакте; TG — только бот-лидмагнит. Письмо пересобрано: «на сайте заявлены YouTube и ВК», без утверждений об отсутствии</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Огромная контентная база и лид-магниты (выкройки, вебинары) без платного трафика; офлайн Мск+СПб + онлайн — идеальный матч под кейс Кинезио || Соцсети: Личный бренд Марии в IG @mari_amochaeva (заблокирован); YouTube + Rutube 514 подборок; VK/TG школы не видны; блог на сайте заброшен (статья 2020 г.)</t>
+          <t>Огромная контентная база и лид-магниты (выкройки, вебинары) без платного трафика; офлайн Мск+СПб + онлайн — идеальный матч под кейс Кинезио || Соцсети: Личный бренд Марии в IG @mari_amochaeva (заблокирован); YouTube + Rutube 514 подборок; VK/TG школы не видны; блог на сайте заброшен (статья 2020 г.) || СОЦРАЗВЕДКА v2 (07.07): ВК — целая живая сеть: vk.com/wanttosew (блог), vk.com/i_want_to_sew_spb, vk.com/wanttosew_msk + vkvideo.ru/@wanttosew; IG @wanttosew ~180K. Письмо пересобрано полностью: сообщества ВК = готовая воронка, оффер — направить на них платный трафик</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Премиум: БЦ Corner Place, врачи из моск. института пластической хирургии, чек до 56 200 ₽ — юнит-экономика Директа сходится с запасом || Соцсети: VK/TG/IG не находятся; ПроДокторов 170 отзывов, 18 врачей</t>
+          <t>Премиум: БЦ Corner Place, врачи из моск. института пластической хирургии, чек до 56 200 ₽ — юнит-экономика Директа сходится с запасом || Соцсети: VK/TG/IG не находятся; ПроДокторов 170 отзывов, 18 врачей || СОЦРАЗВЕДКА v2 (07.07): IG ЕСТЬ — @lancette_nn; ВК не найден (безопасно, но не утверждаем); TG — упоминание в 2ГИС без ссылки. Письмо пересобрано: IG признан активом, «нет ни ВК ни TG» убрано</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2050,7 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис)</t>
+          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис) || СОЦРАЗВЕДКА v2 (07.07): соцсети этой клиники не найдены, НО в Екб есть стоматология-ТЁЗКА «Визави» (centrvizavi.ru, Шейнкмана 9) с ВК/TG — риск перепутать. Письмо пересобрано: «судя по открытым данным» вместо категоричного «канала нет»</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: ВК/TG не видны (Facebook в разведке не учитываем); Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258)</t>
+          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: ВК/TG не видны (Facebook в разведке не учитываем); Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258) || СОЦРАЗВЕДКА v2 (07.07): ВК/TG/IG не найдены ни на сайте, ни поиском (самый чистый кейс), но по правилу «не утверждать отсутствие» формулировка смягчена: «если запись идёт в основном с карт…». Есть заброшенный FB (игнорируем)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 3 send-task queued; unified report refreshed on Drive; newbiz segment: sources methodology, template, 8 first-touch DMs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S26"/>
+  <dimension ref="A1:S42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -909,10 +909,15 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Отправлено</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="n"/>
+          <t>Переговоры</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
@@ -920,7 +925,7 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>С 2009 г.; филиалы у метро Римская и Домодедовская + онлайн-платформа; нет локального платного трафика по районам</t>
+          <t>С 2009 г.; филиалы у метро Римская и Домодедовская + онлайн-платформа; нет локального платного трафика по районам || ПЕРВЫЙ ОТВЕТ КАМПАНИИ (06.07, лаг ~4,5 ч). Интерес: филиал «Римская». Переписку ведёт Яна.</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1314,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Сергей Жучков (основатель, экс-КРОК)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1329,17 +1334,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Родители для ProgKids из Директа</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N12" s="2" t="n"/>
@@ -1350,7 +1355,7 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Резерв: общий support-ящик и международный фокус — письмо на следующий день, если нужен добор квоты</t>
+          <t>Резерв: общий support-ящик и международный фокус — письмо на следующий день, если нужен добор квоты || ДОСЬЕ v2 (07.07): РФ-рынок активен (цены в рублях ~700–900₽/урок, 2ГИС Москва, свежие русские отзывы); основатель Сергей Жучков; партнёрство с МПГУ (Minecraft для учителей); привлекали $1,5M инвестиций; 20 000+ учеников; IG @progkids 21K; ВК упомянут в 2ГИС, URL не подтверждён</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1384,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Аськов Андрей Николаевич (директор и единственный владелец, с 2012)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1399,17 +1404,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Пациенты для нового филиала «Призвания»</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N13" s="2" t="n"/>
@@ -1420,7 +1425,7 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Резерв: семейная многопрофильная клиника, слабее персонализация — дособрать факты перед письмом</t>
+          <t>Резерв: семейная многопрофильная клиника, слабее персонализация — дособрать факты перед письмом || ДОСЬЕ v2 (07.07): 30 врачей, 525 отзывов ПроДокторов, «Лучший медцентр 2023», номинант 2026; локомотивы: гинекология+УЗИ, педиатрия, эндокринология; НОВЫЙ филиал на Владимирской (5 отзывов — раскачать трафиком); ВК/TG не найдены по сниппетам (не подтверждено)</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1506,9 @@
       <c r="B15" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C15" s="2" t="n"/>
+      <c r="C15" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>Клиника врачебной косметологии «Совершенство»</t>
@@ -1549,7 +1556,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N15" s="2" t="n"/>
@@ -1560,7 +1567,7 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>С 2017, аппаратная база InMode; раздел «Акции» на сайте — готовые офферы без трафика; врачи Эльвира Асхатовна, Ляйля Рамиловна || Соцсети: VK/TG не находятся; ПроДокторов 29 положительных отзывов || СОЦРАЗВЕДКА v2 (07.07): сайт заявляет ВК и Telegram (сниппеты контактов); IG @sovershenstvo_clinic. Письмо пересобрано: зацепка на разделе «Акции» без утверждений об отсутствии соцсетей</t>
+          <t>С 2017, аппаратная база InMode; раздел «Акции» на сайте — готовые офферы без трафика; врачи Эльвира Асхатовна, Ляйля Рамиловна || Соцсети: VK/TG не находятся; ПроДокторов 29 положительных отзывов || СОЦРАЗВЕДКА v2 (07.07): сайт заявляет ВК и Telegram (сниппеты контактов); IG @sovershenstvo_clinic. Письмо пересобрано: зацепка на разделе «Акции» без утверждений об отсутствии соцсетей || отправлено 07.07 02:35 UTC — НОВЫЙ черновик; Яна сама сменила тему на «Заявки для «Совершенства»»</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1578,9 @@
       <c r="B16" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C16" s="2" t="n"/>
+      <c r="C16" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>Terra del Sol (центр красоты)</t>
@@ -1619,7 +1628,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N16" s="2" t="n"/>
@@ -1630,7 +1639,7 @@
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
-          <t>19+ лет, 2 филиала (Восход 14/1, пл. К. Маркса); запись только по телефону; устаревший сайт без трафика || Соцсети: VK vk.com/terradelsol; Фламп/2ГИС 4.5 (~130 отзывов), хвалят косметолога Элеонору Винник и стилиста Татьяну Евдокимову</t>
+          <t>19+ лет, 2 филиала (Восход 14/1, пл. К. Маркса); запись только по телефону; устаревший сайт без трафика || Соцсети: VK vk.com/terradelsol; Фламп/2ГИС 4.5 (~130 отзывов), хвалят косметолога Элеонору Винник и стилиста Татьяну Евдокимову || отправлено 07.07 02:44 UTC (корректный черновик от 06.07)</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1650,9 @@
       <c r="B17" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C17" s="2" t="n"/>
+      <c r="C17" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>Салон красоты «Красивые Люди»</t>
@@ -1689,7 +1700,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N17" s="2" t="n"/>
@@ -1700,7 +1711,7 @@
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Полный комплекс услуг; личный gmail директора — короткий цикл сделки; нет онлайн-записи || Соцсети: VK/IG-ссылки на сайте, активного сообщества нет; Zoon/Фламп: хвалят стилиста Мане (Air Touch), мастеров Светлану и Виктора || СОЦРАЗВЕДКА v2 (07.07): yell.ru заявляет VK/IG; вероятный IG @krasivielyudi_official (принадлежность не подтверждена — тёзки в других городах). Письмо пересобрано: убрано «соцсети почти не живут», мягкая формулировка про карты/сарафан</t>
+          <t>Полный комплекс услуг; личный gmail директора — короткий цикл сделки; нет онлайн-записи || Соцсети: VK/IG-ссылки на сайте, активного сообщества нет; Zoon/Фламп: хвалят стилиста Мане (Air Touch), мастеров Светлану и Виктора || СОЦРАЗВЕДКА v2 (07.07): yell.ru заявляет VK/IG; вероятный IG @krasivielyudi_official (принадлежность не подтверждена — тёзки в других городах). Письмо пересобрано: убрано «соцсети почти не живут», мягкая формулировка про карты/сарафан || отправлено 07.07 02:42 UTC — НОВЫЙ черновик (после соцразведки v2)</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1792,9 @@
       <c r="B19" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C19" s="2" t="n"/>
+      <c r="C19" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>Profieng — онлайн-школа английского</t>
@@ -1829,7 +1842,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N19" s="2" t="n"/>
@@ -1840,7 +1853,7 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>IELTS/TOEFL/ЕГЭ + дети 4–12; сезонное окно — набор к учебному году; конкуренты (Skyeng) активно закупают трафик || Соцсети: VK/TG не видны в поиске; 20 отзывов на Kurshub (хвалят цену и расписание); Zoon, 2ГИС || СОЦРАЗВЕДКА v2 (07.07): сайт на странице контактов заявляет YouTube и ВКонтакте; TG — только бот-лидмагнит. Письмо пересобрано: «на сайте заявлены YouTube и ВК», без утверждений об отсутствии</t>
+          <t>IELTS/TOEFL/ЕГЭ + дети 4–12; сезонное окно — набор к учебному году; конкуренты (Skyeng) активно закупают трафик || Соцсети: VK/TG не видны в поиске; 20 отзывов на Kurshub (хвалят цену и расписание); Zoon, 2ГИС || СОЦРАЗВЕДКА v2 (07.07): сайт на странице контактов заявляет YouTube и ВКонтакте; TG — только бот-лидмагнит. Письмо пересобрано: «на сайте заявлены YouTube и ВК», без утверждений об отсутствии || отправлено 07.07 02:37 UTC — УШЛА СТАРАЯ ВЕРСИЯ (формулировка «ВК и TG в поиске почти не видны» — мягкая, риск низкий; сайт ВК заявляет). Новый неотправленный черновик r-1267307485728993365 УДАЛИТЬ. Если ответят про ВК — признать и перевести в пользу: «поэтому и пишем — аудиторию надо развивать рекламой»</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2074,9 @@
       <c r="B23" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C23" s="2" t="n"/>
+      <c r="C23" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>«Центр Стоматологии»</t>
@@ -2109,7 +2124,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N23" s="2" t="n"/>
@@ -2120,7 +2135,7 @@
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: ВК/TG не видны (Facebook в разведке не учитываем); Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258) || СОЦРАЗВЕДКА v2 (07.07): ВК/TG/IG не найдены ни на сайте, ни поиском (самый чистый кейс), но по правилу «не утверждать отсутствие» формулировка смягчена: «если запись идёт в основном с карт…». Есть заброшенный FB (игнорируем)</t>
+          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: ВК/TG не видны (Facebook в разведке не учитываем); Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258) || СОЦРАЗВЕДКА v2 (07.07): ВК/TG/IG не найдены ни на сайте, ни поиском (самый чистый кейс), но по правилу «не утверждать отсутствие» формулировка смягчена: «если запись идёт в основном с карт…». Есть заброшенный FB (игнорируем) || отправлено 07.07 01:55 UTC — НОВЫЙ черновик (v3); Яна сама сменила тему на «Заявки для стоматологий с фиксированной ценой»</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2164,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Анастасия Пяткевич и Алёна Эдигер (сооснователи, ИП Пяткевич А.П.)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2169,17 +2184,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Идея по записям для Timeless</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N24" s="2" t="n"/>
@@ -2190,7 +2205,7 @@
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Резерв: рейтинг ниже конкурентов, нет ЛПР; anti-age авторские методики — фактура для креативов || Соцсети: IG @timeless_studio_massage основной канал; VK не найден; Zoon 3.4; 2 филиала</t>
+          <t>Резерв: рейтинг ниже конкурентов, нет ЛПР; anti-age авторские методики — фактура для креативов || Соцсети: IG @timeless_studio_massage основной канал; VK не найден; Zoon 3.4; 2 филиала || ДОСЬЕ v2 (07.07): email info@timeless-studio.ru подтверждён в сниппетах сайта; сооснователи найдены; сайт делало агентство Chipsa (WebGL) — в упаковку вложились; 3 вакансии на hh — расширяются; открыты 07.2020, Петроградка, 9–22; 2ГИС показывает кнопку ВК (URL не подтверждён)</t>
         </is>
       </c>
     </row>
@@ -2239,17 +2254,17 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Идея для «Триарс» к осеннему набору</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N25" s="2" t="n"/>
@@ -2260,7 +2275,7 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата</t>
+          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата || ДОСЬЕ v2 (07.07): ВК НАЙДЕН — vk.com/triars_school (сниппет Яндекс.Карт); также IG @triars_school, YouTube, Pinterest, TG как канал связи; с 2017; ЛПР не найден (вход через препода Марата); вакансии на hh (employer/3265114) — растут; платной рекламы не видно</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2304,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Сафин Ранас Анасович (гендиректор, совладелец с отцом — семейный бизнес)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2309,17 +2324,17 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Свои пациенты для «21 Век»</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N26" s="2" t="n"/>
@@ -2330,7 +2345,1047 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1</t>
+          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1 || ДОСЬЕ v2 (07.07): ООО «Стоматология XXI век» (ИНН 1660130086, с 2009); акционные лендинги на сайте («кариес 5900₽») — готовы к трафику; ВК/TG не найдены по сниппетам (не подтверждено); одна точка — ЖК «Казань XXI век»</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>LAPLAS — клиника косметологии и пластической хирургии</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Тюмень</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Олейник Евгений Васильевич (гендиректор ООО «Лаплас», с 07.2023)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>info@lap-las.ru</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://lap-las.ru/</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Идея по записям для LAPLAS</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="n"/>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2" t="n"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Yell 5.0 (18), ПроДокторов 48 врачей ~500 отзывов; в отзывах хвалят LPG и Fotona (пигментация за 2 сеанса); с 2018, 7 дней/нед; верх ICP по размеру || Соцсети: IG @laplas_clinic; ВК/TG не найдены по сниппетам (не подтверждено); живут на агрегаторах и картах</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Laser House — клиника лазерной эпиляции и косметологии</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Краснодар</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>laserhousekrd@mail.ru</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://laserhouse23.ru/</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Записи для трёх филиалов Laser House</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n"/>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="2" t="n"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>2ГИС 4.9 (69); MeDioStar NeXT Pro + Asclepion Dermablate; 3 филиала (Краснодар/Туапсе/Новороссийск); онлайн-запись YClients; эстетическая гинекология — маржинальная услуга; ЛПР не найден — уточнить на созвоне || Соцсети: IG laser_house23; ВК/TG не найдены по сниппетам (не подтверждено)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>МиМи|ЛО — студия маникюра и педикюра</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Ростов-на-Дону</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Амосова Мария Алексеевна (ИП, владелица)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ativlasta016@gmail.com</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>personal</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://mimilo-nail.ru/</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Идея по записям для МиМи|ЛО</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="n"/>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="2" t="n"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Яндекс 5.0 при 574 отзывах; «салон в стиле Бали» с бесплатным баром, dog-friendly; акция маникюр+гель-лак 2190₽ — промо уже используют; личный gmail на сайте — короткий цикл сделки || Соцсети: не найдены по сниппетам (не подтверждено)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>iDesign — школа практического дизайна</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Елена и Дмитрий Гринберг (основатели)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>sales.chief@idesign.school</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://idesign.school/</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Студенты для iDesign к осеннему набору</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n"/>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="2" t="n"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>«Первая школа практического дизайна на Урале»; 200+ выпускников/год; 4 направления + детские/подростковые курсы; куратор Ольга Розет (БВШД); центр города (здание УрГАХА), 9–21 ежедневно; email отдела продаж именной || Соцсети: IG @i_design_school; ВК/TG заявлены в карточках, URL не найдены по сниппетам (не подтверждено)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>БьютиМед — клиника эстетической медицины</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Пермь</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Трунова Татьяна Сергеевна (директор и владелица ООО «МЦК «БьютиМед», с 2016)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>b_med59@mail.ru</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://b-med59.ru/</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Идея по записям для «БьютиМед»</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="n"/>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="2" t="n"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>2ГИС 4.9 (544!); ПроДокторов 17 врачей 283 отзыва; 30+ аппаратов, официальная площадка InMode; 2 локации (Советская 26а, Пермская 33); врачебная косметология — высокий чек; SEO развит, платные каналы недожаты || Соцсети: агрегатор указывает ВК/IG, ссылки не подтверждены по сниппетам</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Giovane — центр красоты и молодости</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Уфа</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Галиханова Лилия Илдусовна (директор и главврач)</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>contact@giovane-clinic.ru</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://giovane-clinic.ru/</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n"/>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="2" t="n"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Резерв (верхняя граница ICP — крупный): Яндекс 4.8 (227); 3 этажа, 1500+ услуг, 2 адреса; активны на скидочных агрегаторах (СКИДКОМ, Lovefit) — платят за лидов, аргумент пересадить бюджет на ВК/Директ || Соцсети: 2ГИС показывает кнопки ВК/WA/TG, URL не подтверждены</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>МузКласс — школа современной музыки</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Нижний Новгород</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Погодин Василий Александрович (директор ООО «МУЗКЛАСС»)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>muzclass@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>http://muzclass.com/</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="n"/>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="2" t="n"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Резерв: с 2016; вокал/гитара/барабаны/фортепиано/скрипка — много сегментов; 2 адреса в каталогах; конкурируют с федеральными сетями («Виртуозы», «Не Школа») || Соцсети: ВК vk.com/club113992055 (вероятно малоактивен); IG @muzclassnn; TG не найден</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Родная клиника — медцентр</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Ростов-на-Дону</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Родной Андрей Юрьевич (директор ООО «ЦДМ» — ФИО требует проверки); главврач Зеньков А. М. (гинеколог)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>rodnay.clinica@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://rodnayklinikarostov.ru/</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n"/>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="2" t="n"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Резерв: ПроДокторов 24 врача, 1570 отзывов; локомотив гинекология; раздел /landings/ на сайте — посадочные под платный трафик уже пробуют; одна точка на Ворошиловском || Соцсети: на сайте кнопки ВК/TG/WA, URL не подтверждены</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>RAFIREL — премиум-салон красоты</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Тюмень</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://rafirel.ru</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="n"/>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="2" t="n"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>НОВИЧОК: открыт ~11.2025 (лонгрид 72.ru 12.03.2026); топ-10 Народной премии 72.RU; 5.0 и 178 отзывов 2ГИС; 2 основателя; уже платят за PR — бюджет есть || Телефон: +7 909 191-10-90</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Stomberry — стоматология (клиника на Комсомольской)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Тюмень</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://www.stomberry.ru</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n"/>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="2" t="n"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>НОВИЧОК: премия 2ГИС «Открытие года»-2026 (младше 6 мес); 2-я клиника сети (1-я на Широтной); имплантация/КТ/седация/детский приём; рейтинг Startsmile-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Академия VIP Beauty — центр медицины и красоты</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Нижний Новгород</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://academy-vip.com</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="n"/>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="2" t="n"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>НОВИЧОК: новость NN.RU об открытии (Алексеевская 10/16, галерея LP Fashion); филиал сети «Академия VIP» (10+ лет); лазерное омоложение, контурная пластика; месяц статьи уточнить || Телефон: 414-88-44</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Лювиталь — клиника детокса, долголетия и красоты</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Кольцово (Новосибирск)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://luvital.ru</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n"/>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="2" t="n"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>НОВИЧОК: открыта весной 2025 (kolcovo.ru, ЧС-ИНФО 26.03.2025); финалист «Открытие года» НГС-2026; SPA-капсулы, водородная терапия; нужен трафик из Нска — гео-таргет || Телефон: +7 923 000-09-85</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Хвоя Сити — премиум-термы и СПА</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://hvoya-city.ru</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="n"/>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="2" t="n"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>НОВИЧОК: победитель «Открытие года» Народной премии НГС-2026; СПА/массаж/аромапарения; ёмкость по абонементам — системный маркетинг || Телефон: 8 383 209-21-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Точка Красоты — 26-й салон сети (франшиза)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Краснодар</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://tochkafamily.ru</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n"/>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="2" t="n"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>НОВИЧОК: новость на сайте сети об открытии в ТЦ «Красная Площадь» (Дзержинского 100); ЛПР — франчайзи, юрлицо искать в Rusprofile по адресу; дата публикации новости — проверить || Телефон: 8 928 464-88-80</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Мега-Дент — новый центр имплантации (Герцена 55)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Тюмень</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://mega-dent72.ru</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="n"/>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="2" t="n"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>НОВИЧОК (неподтверждено): филиал заявлен как новый на сайте сети; сеть — Startsmile TOP 2026 (Forbes); All-on-4/6 — дорогой сегмент; ПЕРЕД касанием подтвердить дату открытия</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>KIBERone — детская школа программирования (филиал Мурино)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Мурино (СПб)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://spb-kudrovo.kiber-one.com</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n"/>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="2" t="n"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>НОВИЧОК (год открытия подтвердить, вероятно 12.2025): франшизный филиал на шоссе Лаврики; набор групп к сентябрю — сезонная боль; ЛПР — франчайзи</t>
         </is>
       </c>
     </row>
@@ -2345,7 +3400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2372,7 +3427,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -2382,7 +3437,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -2402,7 +3457,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -2422,7 +3477,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -2432,7 +3487,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2442,7 +3497,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>0</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="11">
@@ -2452,7 +3507,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -2556,7 +3611,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -2581,7 +3636,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -2606,16 +3661,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -2671,193 +3726,243 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>По типу ящика</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Сегмент</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>Отправлено</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>Bounce</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>Ответов</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>Reply rate</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>Созвонов</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>Конверсия</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>14</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>personal</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>По наличию имени ЛПР</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Сегмент</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>Отправлено</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>Bounce</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>Ответов</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>Reply rate</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>Созвонов</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>Конверсия</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>без имени</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
         <v>10</v>
       </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>По типу ящика</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>Сегмент</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
-        <is>
-          <t>Отправлено</t>
-        </is>
-      </c>
-      <c r="C30" s="1" t="inlineStr">
-        <is>
-          <t>Bounce</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="inlineStr">
-        <is>
-          <t>Ответов</t>
-        </is>
-      </c>
-      <c r="E30" s="1" t="inlineStr">
-        <is>
-          <t>Reply rate</t>
-        </is>
-      </c>
-      <c r="F30" s="1" t="inlineStr">
-        <is>
-          <t>Созвонов</t>
-        </is>
-      </c>
-      <c r="G30" s="1" t="inlineStr">
-        <is>
-          <t>Конверсия</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>generic</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>10</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>По наличию имени ЛПР</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>Сегмент</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="inlineStr">
-        <is>
-          <t>Отправлено</t>
-        </is>
-      </c>
-      <c r="C34" s="1" t="inlineStr">
-        <is>
-          <t>Bounce</t>
-        </is>
-      </c>
-      <c r="D34" s="1" t="inlineStr">
-        <is>
-          <t>Ответов</t>
-        </is>
-      </c>
-      <c r="E34" s="1" t="inlineStr">
-        <is>
-          <t>Reply rate</t>
-        </is>
-      </c>
-      <c r="F34" s="1" t="inlineStr">
-        <is>
-          <t>Созвонов</t>
-        </is>
-      </c>
-      <c r="G34" s="1" t="inlineStr">
-        <is>
-          <t>Конверсия</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>без имени</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>7</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>имя известно</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>3</v>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>Ориентиры (источник — playbook.md, «Ориентиры метрик» и «Ворота выборки»): reply rate 3–7% норма, &lt;2% при ≥50 доставленных — тревога; bounce &gt;5% — тревога; тема/абзац — только по A/B ≥40 отправок на вариант; отказ от ниши — 0 ответов на 60 отправках или (bounce+отписки) &gt;15%; пересмотр базы — отписки+жалобы ≥8. Решения — только по дозревшим когортам ≥14 дней (лист 3) и через подтверждение Яны.</t>
         </is>
@@ -2960,28 +4065,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>0</v>
+        <v>0.0667</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -3054,13 +4159,13 @@
         <v>46209</v>
       </c>
       <c r="B2" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Dental deck: save to assets, rebuild Vizavi & 21 Vek drafts with attachment line, rule in template (Yana attaches file manually)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -2063,7 +2063,7 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис) || СОЦРАЗВЕДКА v2 (07.07): соцсети этой клиники не найдены, НО в Екб есть стоматология-ТЁЗКА «Визави» (centrvizavi.ru, Шейнкмана 9) с ВК/TG — риск перепутать. Письмо пересобрано: «судя по открытым данным» вместо категоричного «канала нет»</t>
+          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис) || СОЦРАЗВЕДКА v2 (07.07): соцсети этой клиники не найдены, НО в Екб есть стоматология-ТЁЗКА «Визави» (centrvizavi.ru, Шейнкмана 9) с ВК/TG — риск перепутать. Письмо пересобрано: «судя по открытым данным» вместо категоричного «канала нет» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v3 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r-5266668500978660320 удалить</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: ВК/TG не видны (Facebook в разведке не учитываем); Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258) || СОЦРАЗВЕДКА v2 (07.07): ВК/TG/IG не найдены ни на сайте, ни поиском (самый чистый кейс), но по правилу «не утверждать отсутствие» формулировка смягчена: «если запись идёт в основном с карт…». Есть заброшенный FB (игнорируем) || отправлено 07.07 01:55 UTC — НОВЫЙ черновик (v3); Яна сама сменила тему на «Заявки для стоматологий с фиксированной ценой»</t>
+          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: ВК/TG не видны (Facebook в разведке не учитываем); Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258) || СОЦРАЗВЕДКА v2 (07.07): ВК/TG/IG не найдены ни на сайте, ни поиском (самый чистый кейс), но по правилу «не утверждать отсутствие» формулировка смягчена: «если запись идёт в основном с карт…». Есть заброшенный FB (игнорируем) || отправлено 07.07 01:55 UTC — НОВЫЙ черновик (v3); Яна сама сменила тему на «Заявки для стоматологий с фиксированной ценой» || ПРЕЗЕНТАЦИЯ: холодное письмо ушло 07.07 без вложения — приложить «OMG-кейсы-стоматологии.pptx» к фоллоу-апу D+3 (10.07), это сильный повод для второго касания</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2345,7 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1 || ДОСЬЕ v2 (07.07): ООО «Стоматология XXI век» (ИНН 1660130086, с 2009); акционные лендинги на сайте («кариес 5900₽») — готовы к трафику; ВК/TG не найдены по сниппетам (не подтверждено); одна точка — ЖК «Казань XXI век»</t>
+          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1 || ДОСЬЕ v2 (07.07): ООО «Стоматология XXI век» (ИНН 1660130086, с 2009); акционные лендинги на сайте («кариес 5900₽») — готовы к трафику; ВК/TG не найдены по сниппетам (не подтверждено); одна точка — ЖК «Казань XXI век» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v2 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r5373719259897128450 удалить</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 4: 10 drafts with social-links signature (user-directed same-day batch), 5 new reserves, Asana task created
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2744,17 +2744,17 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Идея по записям для Giovane</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N32" s="2" t="n"/>
@@ -2765,7 +2765,7 @@
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Резерв (верхняя граница ICP — крупный): Яндекс 4.8 (227); 3 этажа, 1500+ услуг, 2 адреса; активны на скидочных агрегаторах (СКИДКОМ, Lovefit) — платят за лидов, аргумент пересадить бюджет на ВК/Директ || Соцсети: 2ГИС показывает кнопки ВК/WA/TG, URL не подтверждены</t>
+          <t>Резерв (верхняя граница ICP — крупный): Яндекс 4.8 (227); 3 этажа, 1500+ услуг, 2 адреса; активны на скидочных агрегаторах (СКИДКОМ, Lovefit) — платят за лидов, аргумент пересадить бюджет на ВК/Директ || Соцсети: 2ГИС показывает кнопки ВК/WA/TG, URL не подтверждены || ПРОВЕРКА 07.07: email подтверждён (+ запасной team@giovane-clinic.ru); 2ГИС 4.6/442; ПроДокторов 25 врачей; APTOS-сертификация</t>
         </is>
       </c>
     </row>
@@ -2814,17 +2814,17 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ученики для МузКласса из ВКонтакте</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N33" s="2" t="n"/>
@@ -2835,7 +2835,7 @@
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Резерв: с 2016; вокал/гитара/барабаны/фортепиано/скрипка — много сегментов; 2 адреса в каталогах; конкурируют с федеральными сетями («Виртуозы», «Не Школа») || Соцсети: ВК vk.com/club113992055 (вероятно малоактивен); IG @muzclassnn; TG не найден</t>
+          <t>Резерв: с 2016; вокал/гитара/барабаны/фортепиано/скрипка — много сегментов; 2 адреса в каталогах; конкурируют с федеральными сетями («Виртуозы», «Не Школа») || Соцсети: ВК vk.com/club113992055 (вероятно малоактивен); IG @muzclassnn; TG не найден || ПРОВЕРКА 07.07: школа жива, уже 3 адреса (расширение!); email актуален; актуальный ВК vk.com/muzclasscom; урок 60 мин — дифференциатор</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Родной Андрей Юрьевич (директор ООО «ЦДМ» — ФИО требует проверки); главврач Зеньков А. М. (гинеколог)</t>
+          <t>Родной Андрей Юрьевич (директор и учредитель ООО «ЦДМ» — подтверждено); главврач Зеньков А.М.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2884,17 +2884,17 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Пациентки для «Родной клиники»</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N34" s="2" t="n"/>
@@ -2905,7 +2905,7 @@
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Резерв: ПроДокторов 24 врача, 1570 отзывов; локомотив гинекология; раздел /landings/ на сайте — посадочные под платный трафик уже пробуют; одна точка на Ворошиловском || Соцсети: на сайте кнопки ВК/TG/WA, URL не подтверждены</t>
+          <t>Резерв: ПроДокторов 24 врача, 1570 отзывов; локомотив гинекология; раздел /landings/ на сайте — посадочные под платный трафик уже пробуют; одна точка на Ворошиловском || Соцсети: на сайте кнопки ВК/TG/WA, URL не подтверждены || ПРОВЕРКА 07.07: директор ПОДТВЕРЖДЁН — Родной Андрей Юрьевич (учредитель ООО «ЦДМ», checko); email актуален (ya.ru = алиас yandex.ru)</t>
         </is>
       </c>
     </row>
@@ -3386,6 +3386,846 @@
       <c r="S42" t="inlineStr">
         <is>
           <t>НОВИЧОК (год открытия подтвердить, вероятно 12.2025): франшизный филиал на шоссе Лаврики; набор групп к сентябрю — сезонная боль; ЛПР — франчайзи</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Face &amp; Body — клиника косметологии и гинекологии</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Красноярск</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>klinika@facebody.ru</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://facebody.ru/</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Идея по записям для Face &amp; Body</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="n"/>
+      <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="2" t="n"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>«Нимфа» — сеть салонов красоты (4 точки)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Омск</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Трутнева Татьяна Анатольевна (директор ООО «СК «Нимфа» с 2008)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>marketingnimfa@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://salon-nimfa.ru/</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Записи для четырёх салонов «Нимфы»</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="n"/>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="2" t="n"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Сеть 4 салона; 4.6/140 2ГИС; премиум аппаратная+инъекционная косметология, лазерная эпиляция; ВЫДЕЛЕННЫЙ маркетинговый email (пишем на него); осн. ящик nimfa2002@bk.ru || Соцсети: IG @nimfa_omsk; ВК кнопка на картах, URL не подтверждён</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>SOHO — салон красоты и косметологии (3 филиала)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Воронеж</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Камышников Сергей Анатольевич (директор ООО «СОХО»)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>soho@list.ru</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://salonsoho.ru/</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Идея по записям для SOHO</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="n"/>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="2" t="n"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>С 2005, 26 сотрудников; 3 филиала вкл. ТЦ «Галерея Чижова»; отдельная косметологическая клиника (cosmetology-voronezh.ru, 6 врачей, 45 отзывов ПроДокторов) || Соцсети: ВК/TG упомянуты в 2ГИС, URL не подтверждены</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Lingua City — языковая школа</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Красноярск</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Локтионова Татьяна Александровна (директор)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>lingua.city@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://linguacity-school.ru/</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Ученики для Lingua City к сентябрю</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="n"/>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="2" t="n"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>2 филиала (Ястынская 7, Карамзина 13); Zoon 4.3; ученики занимаются 3–6 лет (высокий LTV); есть промо-лендинг promo.linguacity-school.ru — уже вкладываются в трафик || Соцсети: не найдены по сниппетам (не подтверждено)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>«Живой Язык» — языковая школа</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Тюмень</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Бауэр Виктория Юрьевна (директор)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>info@livlang.ru</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://livlang.ru/</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Набор к сентябрю для «Живого Языка»</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="n"/>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="2" t="n"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>С 1998, лицензированная; 3 локации; IELTS/TOEFL/FCE + ЕГЭ/ОГЭ + обучение за рубежом (высокий чек); рейтинг лучших школ города (1tmn.ru) || Соцсети: ВК vk.com/livinglanguage (подтверждён), IG @living_language; TG не найден</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>«Клиника в Северном» + «Первый частный травмпункт»</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Красноярск</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Арбатская Евгения Михайловна (директор); главврач Акуленко Мария Олеговна</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>clients@clinsev.ru</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>http://clinsev.ru/</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Пациенты для «Клиники в Северном»</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="n"/>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="2" t="n"/>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>56 врачей, 851 отзыв ПроДокторов; УНИКУМ: единственный в городе частный круглосуточный травмпункт — готовый оффер для Директа; агрегаторная зависимость (ПроДокторов/Фламп/Zoon/DocDoc) || Соцсети: ВК заявлен в orgpage, URL не подтверждён</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>«Докториус» (экс-«Авиценна») — клиника</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Ижевск</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Розов Александр Николаевич (директор и учредитель 38% ООО «Авиценна»)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>avicenna18@mail.ru</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://doktorius.ru/</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Пациенты на новое имя «Докториус»</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="n"/>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="2" t="n"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>РЕБРЕНДИНГ Авиценна→Докториус — повод касания: новое имя надо прогревать рекламой; 45 врачей, 1232 отзыва ПроДокторов; email ещё старый avicenna18@ || Соцсети: ВК vk.com/doktorius_klinica</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>«Ренессанс плюс» — частная школа искусств</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Омск</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Остапенко Елена Анатольевна (директор)</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>art635068@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://www.renaissance55.ru/</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="n"/>
+      <c r="P50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="2" t="n"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Резерв: с 2012, 1400+ учеников, 12 направлений (вокал/инструменты/живопись/актёрское); взрослые И дети 5+; концерты — готовый контент; слабое соцприсутствие</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Uclinic — клиника экспертной косметологии</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Волгоград</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Емельянов Андрей Павлович (директор и основатель, тренер Merz Aesthetics)</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>info@u-clinic.ru</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://u-clinic.ru/</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="n"/>
+      <c r="P51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="2" t="n"/>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Резерв: премии ПроДокторов 2020/2021/2023, 498 отзывов, 14 врачей; своё приложение записи; InMode; направление «Косметология до 25 / Glow Club»; сильный собственный маркетинг — калибровать оффер || IG @uclinic.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>«АртМед» — сеть медцентров (реабилитация/ЦВЛ)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Омск</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Филимендиков Павел Владимирович (директор ООО «МЦ «Артмед +» — юрлиц несколько, аккуратно)</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>artmed555@mail.ru</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://artmed55.ru/</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="n"/>
+      <c r="P52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="2" t="n"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Резерв: 3–4 филиала, 107 врачей, 890 отзывов ПроДокторов; локомотив — восстановительное лечение; ВК vk.com/cvl55 (старое имя — соцсети запущены); запасной email info@artmedomsk.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>«Пересвет» — медцентр (4 филиала, КТ/МРТ)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Воронеж</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Агафонова Ирина Сергеевна (главврач)</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>mail@peresvet.vrn.ru</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://mc-peresvet.ru/</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="n"/>
+      <c r="P53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="2" t="n"/>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Резерв (верх ICP): 4 филиала + стационар, 47 врачей, 342 отзыва ПроДокторов, КТ/МРТ/пластика || Соцсети: ВК/TG заявлены на сайте, URL не подтверждены</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Essenti — врачебная косметология</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Волгоград</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Веремеенко Владимир Валентинович (гендиректор)</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>essenti34@gmail.com</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://essenti.ru/</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="n"/>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="2" t="n"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Резерв на будущее (не дублировать Волгоград с Uclinic в одном батче)</t>
         </is>
       </c>
     </row>
@@ -3427,7 +4267,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -3437,7 +4277,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -4159,7 +4999,7 @@
         <v>46209</v>
       </c>
       <c r="B2" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C2" t="n">
         <v>15</v>

</xml_diff>

<commit_message>
Batch 4 v2: HTML letters with hyperlinks, copy-edit pass, Doktorius fact fixed (name since 2023); new rules: date verification, sales/language checklist
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -2765,7 +2765,7 @@
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Резерв (верхняя граница ICP — крупный): Яндекс 4.8 (227); 3 этажа, 1500+ услуг, 2 адреса; активны на скидочных агрегаторах (СКИДКОМ, Lovefit) — платят за лидов, аргумент пересадить бюджет на ВК/Директ || Соцсети: 2ГИС показывает кнопки ВК/WA/TG, URL не подтверждены || ПРОВЕРКА 07.07: email подтверждён (+ запасной team@giovane-clinic.ru); 2ГИС 4.6/442; ПроДокторов 25 врачей; APTOS-сертификация</t>
+          <t>Резерв (верхняя граница ICP — крупный): Яндекс 4.8 (227); 3 этажа, 1500+ услуг, 2 адреса; активны на скидочных агрегаторах (СКИДКОМ, Lovefit) — платят за лидов, аргумент пересадить бюджет на ВК/Директ || Соцсети: 2ГИС показывает кнопки ВК/WA/TG, URL не подтверждены || ПРОВЕРКА 07.07: email подтверждён (+ запасной team@giovane-clinic.ru); 2ГИС 4.6/442; ПроДокторов 25 врачей; APTOS-сертификация || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2835,7 @@
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Резерв: с 2016; вокал/гитара/барабаны/фортепиано/скрипка — много сегментов; 2 адреса в каталогах; конкурируют с федеральными сетями («Виртуозы», «Не Школа») || Соцсети: ВК vk.com/club113992055 (вероятно малоактивен); IG @muzclassnn; TG не найден || ПРОВЕРКА 07.07: школа жива, уже 3 адреса (расширение!); email актуален; актуальный ВК vk.com/muzclasscom; урок 60 мин — дифференциатор</t>
+          <t>Резерв: с 2016; вокал/гитара/барабаны/фортепиано/скрипка — много сегментов; 2 адреса в каталогах; конкурируют с федеральными сетями («Виртуозы», «Не Школа») || Соцсети: ВК vk.com/club113992055 (вероятно малоактивен); IG @muzclassnn; TG не найден || ПРОВЕРКА 07.07: школа жива, уже 3 адреса (расширение!); email актуален; актуальный ВК vk.com/muzclasscom; урок 60 мин — дифференциатор || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Резерв: ПроДокторов 24 врача, 1570 отзывов; локомотив гинекология; раздел /landings/ на сайте — посадочные под платный трафик уже пробуют; одна точка на Ворошиловском || Соцсети: на сайте кнопки ВК/TG/WA, URL не подтверждены || ПРОВЕРКА 07.07: директор ПОДТВЕРЖДЁН — Родной Андрей Юрьевич (учредитель ООО «ЦДМ», checko); email актуален (ya.ru = алиас yandex.ru)</t>
+          <t>Резерв: ПроДокторов 24 врача, 1570 отзывов; локомотив гинекология; раздел /landings/ на сайте — посадочные под платный трафик уже пробуют; одна точка на Ворошиловском || Соцсети: на сайте кнопки ВК/TG/WA, URL не подтверждены || ПРОВЕРКА 07.07: директор ПОДТВЕРЖДЁН — Родной Андрей Юрьевич (учредитель ООО «ЦДМ», checko); email актуален (ya.ru = алиас yandex.ru) || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3455,7 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены</t>
+          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Сеть 4 салона; 4.6/140 2ГИС; премиум аппаратная+инъекционная косметология, лазерная эпиляция; ВЫДЕЛЕННЫЙ маркетинговый email (пишем на него); осн. ящик nimfa2002@bk.ru || Соцсети: IG @nimfa_omsk; ВК кнопка на картах, URL не подтверждён</t>
+          <t>Сеть 4 салона; 4.6/140 2ГИС; премиум аппаратная+инъекционная косметология, лазерная эпиляция; ВЫДЕЛЕННЫЙ маркетинговый email (пишем на него); осн. ящик nimfa2002@bk.ru || Соцсети: IG @nimfa_omsk; ВК кнопка на картах, URL не подтверждён || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr">
         <is>
-          <t>С 2005, 26 сотрудников; 3 филиала вкл. ТЦ «Галерея Чижова»; отдельная косметологическая клиника (cosmetology-voronezh.ru, 6 врачей, 45 отзывов ПроДокторов) || Соцсети: ВК/TG упомянуты в 2ГИС, URL не подтверждены</t>
+          <t>С 2005, 26 сотрудников; 3 филиала вкл. ТЦ «Галерея Чижова»; отдельная косметологическая клиника (cosmetology-voronezh.ru, 6 врачей, 45 отзывов ПроДокторов) || Соцсети: ВК/TG упомянуты в 2ГИС, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
-          <t>2 филиала (Ястынская 7, Карамзина 13); Zoon 4.3; ученики занимаются 3–6 лет (высокий LTV); есть промо-лендинг promo.linguacity-school.ru — уже вкладываются в трафик || Соцсети: не найдены по сниппетам (не подтверждено)</t>
+          <t>2 филиала (Ястынская 7, Карамзина 13); Zoon 4.3; ученики занимаются 3–6 лет (высокий LTV); есть промо-лендинг promo.linguacity-school.ru — уже вкладываются в трафик || Соцсети: не найдены по сниппетам (не подтверждено) || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
-          <t>С 1998, лицензированная; 3 локации; IELTS/TOEFL/FCE + ЕГЭ/ОГЭ + обучение за рубежом (высокий чек); рейтинг лучших школ города (1tmn.ru) || Соцсети: ВК vk.com/livinglanguage (подтверждён), IG @living_language; TG не найден</t>
+          <t>С 1998, лицензированная; 3 локации; IELTS/TOEFL/FCE + ЕГЭ/ОГЭ + обучение за рубежом (высокий чек); рейтинг лучших школ города (1tmn.ru) || Соцсети: ВК vk.com/livinglanguage (подтверждён), IG @living_language; TG не найден || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -3805,7 +3805,7 @@
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr">
         <is>
-          <t>56 врачей, 851 отзыв ПроДокторов; УНИКУМ: единственный в городе частный круглосуточный травмпункт — готовый оффер для Директа; агрегаторная зависимость (ПроДокторов/Фламп/Zoon/DocDoc) || Соцсети: ВК заявлен в orgpage, URL не подтверждён</t>
+          <t>56 врачей, 851 отзыв ПроДокторов; УНИКУМ: единственный в городе частный круглосуточный травмпункт — готовый оффер для Директа; агрегаторная зависимость (ПроДокторов/Фламп/Zoon/DocDoc) || Соцсети: ВК заявлен в orgpage, URL не подтверждён || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Пациенты на новое имя «Докториус»</t>
+          <t>Свои пациенты для «Докториуса»</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3875,7 +3875,7 @@
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr">
         <is>
-          <t>РЕБРЕНДИНГ Авиценна→Докториус — повод касания: новое имя надо прогревать рекламой; 45 врачей, 1232 отзыва ПроДокторов; email ещё старый avicenna18@ || Соцсети: ВК vk.com/doktorius_klinica</t>
+          <t>ФАКТ-ЧЕК Яны 07.07: название «Докториус» используется минимум с 2023 (отзывы за май/сент/ноябрь 2023) — НЕ свежий ребрендинг, зацепка исправлена на «отзывная база + собственный канал»; 45 врачей, 1232 отзыва ПроДокторов; email ещё старый avicenna18@ || Соцсети: ВК vk.com/doktorius_klinica || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ban scripted CTA phrase per Yana; rebuild 7 unsent variant-A drafts (HTML, new CTA); reconcile sends 07-08.07; iDesign polite refusal -> not_interested
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -1366,7 +1366,9 @@
       <c r="B13" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C13" s="2" t="n"/>
+      <c r="C13" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>Клиника «Призвание»</t>
@@ -1414,7 +1416,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N13" s="2" t="n"/>
@@ -1425,7 +1427,7 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Резерв: семейная многопрофильная клиника, слабее персонализация — дособрать факты перед письмом || ДОСЬЕ v2 (07.07): 30 врачей, 525 отзывов ПроДокторов, «Лучший медцентр 2023», номинант 2026; локомотивы: гинекология+УЗИ, педиатрия, эндокринология; НОВЫЙ филиал на Владимирской (5 отзывов — раскачать трафиком); ВК/TG не найдены по сниппетам (не подтверждено)</t>
+          <t>Резерв: семейная многопрофильная клиника, слабее персонализация — дособрать факты перед письмом || ДОСЬЕ v2 (07.07): 30 врачей, 525 отзывов ПроДокторов, «Лучший медцентр 2023», номинант 2026; локомотивы: гинекология+УЗИ, педиатрия, эндокринология; НОВЫЙ филиал на Владимирской (5 отзывов — раскачать трафиком); ВК/TG не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:43 UTC</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1497,7 @@
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>16 лет, ТОП-клиник Сибири 2023; широкая линейка (лазер, вес, подология, трихология); брендовый спрос уходит агрегаторам || Соцсети: VK указан в контактах, но не находится в поиске; 2ГИС 4.7 (302 оценки); негатив — про администраторов || СОЦРАЗВЕДКА v2 (07.07, после ошибки): ВК ЕСТЬ — vk.com/altikansk (подтверждено Яной; сайт заявляет ВК/WhatsApp/TG, страница ВК не индексируется поиском). Письмо пересобрано: зацепка на репутации+ВК, утверждение об отсутствии убрано</t>
+          <t>16 лет, ТОП-клиник Сибири 2023; широкая линейка (лазер, вес, подология, трихология); брендовый спрос уходит агрегаторам || Соцсети: VK указан в контактах, но не находится в поиске; 2ГИС 4.7 (302 оценки); негатив — про администраторов || СОЦРАЗВЕДКА v2 (07.07, после ошибки): ВК ЕСТЬ — vk.com/altikansk (подтверждено Яной; сайт заявляет ВК/WhatsApp/TG, страница ВК не индексируется поиском). Письмо пересобрано: зацепка на репутации+ВК, утверждение об отсутствии убрано || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1783,7 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3 || СОЦРАЗВЕДКА v2 (07.07): Telegram-канал ЕСТЬ — t.me/naydisebyamsk; IG @naydisebya_ru 8,2K + @naydisebya.online; ВК не найден по сниппетам (не подтверждено). Письмо пересобрано: TG признан активом, утверждение «TG не развит» убрано</t>
+          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3 || СОЦРАЗВЕДКА v2 (07.07): Telegram-канал ЕСТЬ — t.me/naydisebyamsk; IG @naydisebya_ru 8,2K + @naydisebya.online; ВК не найден по сниппетам (не подтверждено). Письмо пересобрано: TG признан активом, утверждение «TG не развит» убрано || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1925,7 @@
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Огромная контентная база и лид-магниты (выкройки, вебинары) без платного трафика; офлайн Мск+СПб + онлайн — идеальный матч под кейс Кинезио || Соцсети: Личный бренд Марии в IG @mari_amochaeva (заблокирован); YouTube + Rutube 514 подборок; VK/TG школы не видны; блог на сайте заброшен (статья 2020 г.) || СОЦРАЗВЕДКА v2 (07.07): ВК — целая живая сеть: vk.com/wanttosew (блог), vk.com/i_want_to_sew_spb, vk.com/wanttosew_msk + vkvideo.ru/@wanttosew; IG @wanttosew ~180K. Письмо пересобрано полностью: сообщества ВК = готовая воронка, оффер — направить на них платный трафик</t>
+          <t>Огромная контентная база и лид-магниты (выкройки, вебинары) без платного трафика; офлайн Мск+СПб + онлайн — идеальный матч под кейс Кинезио || Соцсети: Личный бренд Марии в IG @mari_amochaeva (заблокирован); YouTube + Rutube 514 подборок; VK/TG школы не видны; блог на сайте заброшен (статья 2020 г.) || СОЦРАЗВЕДКА v2 (07.07): ВК — целая живая сеть: vk.com/wanttosew (блог), vk.com/i_want_to_sew_spb, vk.com/wanttosew_msk + vkvideo.ru/@wanttosew; IG @wanttosew ~180K. Письмо пересобрано полностью: сообщества ВК = готовая воронка, оффер — направить на них платный трафик || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2006,9 @@
       <c r="B22" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C22" s="2" t="n"/>
+      <c r="C22" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>Стоматологическая клиника «Визави»</t>
@@ -2052,7 +2056,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N22" s="2" t="n"/>
@@ -2063,7 +2067,7 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис) || СОЦРАЗВЕДКА v2 (07.07): соцсети этой клиники не найдены, НО в Екб есть стоматология-ТЁЗКА «Визави» (centrvizavi.ru, Шейнкмана 9) с ВК/TG — риск перепутать. Письмо пересобрано: «судя по открытым данным» вместо категоричного «канала нет» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v3 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r-5266668500978660320 удалить</t>
+          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис) || СОЦРАЗВЕДКА v2 (07.07): соцсети этой клиники не найдены, НО в Екб есть стоматология-ТЁЗКА «Визави» (centrvizavi.ru, Шейнкмана 9) с ВК/TG — риск перепутать. Письмо пересобрано: «судя по открытым данным» вместо категоричного «канала нет» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v3 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r-5266668500978660320 удалить || отправлено 07.07 04:50 UTC — v3 с презентацией</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2279,7 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата || ДОСЬЕ v2 (07.07): ВК НАЙДЕН — vk.com/triars_school (сниппет Яндекс.Карт); также IG @triars_school, YouTube, Pinterest, TG как канал связи; с 2017; ЛПР не найден (вход через препода Марата); вакансии на hh (employer/3265114) — растут; платной рекламы не видно</t>
+          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата || ДОСЬЕ v2 (07.07): ВК НАЙДЕН — vk.com/triars_school (сниппет Яндекс.Карт); также IG @triars_school, YouTube, Pinterest, TG как канал связи; с 2017; ЛПР не найден (вход через препода Марата); вакансии на hh (employer/3265114) — растут; платной рекламы не видно || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2419,7 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Yell 5.0 (18), ПроДокторов 48 врачей ~500 отзывов; в отзывах хвалят LPG и Fotona (пигментация за 2 сеанса); с 2018, 7 дней/нед; верх ICP по размеру || Соцсети: IG @laplas_clinic; ВК/TG не найдены по сниппетам (не подтверждено); живут на агрегаторах и картах</t>
+          <t>Yell 5.0 (18), ПроДокторов 48 врачей ~500 отзывов; в отзывах хвалят LPG и Fotona (пигментация за 2 сеанса); с 2018, 7 дней/нед; верх ICP по размеру || Соцсети: IG @laplas_clinic; ВК/TG не найдены по сниппетам (не подтверждено); живут на агрегаторах и картах || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2430,9 @@
       <c r="B28" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C28" s="2" t="n"/>
+      <c r="C28" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>Laser House — клиника лазерной эпиляции и косметологии</t>
@@ -2474,7 +2480,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N28" s="2" t="n"/>
@@ -2485,7 +2491,7 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
-          <t>2ГИС 4.9 (69); MeDioStar NeXT Pro + Asclepion Dermablate; 3 филиала (Краснодар/Туапсе/Новороссийск); онлайн-запись YClients; эстетическая гинекология — маржинальная услуга; ЛПР не найден — уточнить на созвоне || Соцсети: IG laser_house23; ВК/TG не найдены по сниппетам (не подтверждено)</t>
+          <t>2ГИС 4.9 (69); MeDioStar NeXT Pro + Asclepion Dermablate; 3 филиала (Краснодар/Туапсе/Новороссийск); онлайн-запись YClients; эстетическая гинекология — маржинальная услуга; ЛПР не найден — уточнить на созвоне || Соцсети: IG laser_house23; ВК/TG не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:39 UTC</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2502,9 @@
       <c r="B29" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C29" s="2" t="n"/>
+      <c r="C29" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>МиМи|ЛО — студия маникюра и педикюра</t>
@@ -2544,7 +2552,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N29" s="2" t="n"/>
@@ -2555,7 +2563,7 @@
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Яндекс 5.0 при 574 отзывах; «салон в стиле Бали» с бесплатным баром, dog-friendly; акция маникюр+гель-лак 2190₽ — промо уже используют; личный gmail на сайте — короткий цикл сделки || Соцсети: не найдены по сниппетам (не подтверждено)</t>
+          <t>Яндекс 5.0 при 574 отзывах; «салон в стиле Бали» с бесплатным баром, dog-friendly; акция маникюр+гель-лак 2190₽ — промо уже используют; личный gmail на сайте — короткий цикл сделки || Соцсети: не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:41 UTC (старый CTA-A — уже в поле)</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2574,9 @@
       <c r="B30" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C30" s="2" t="n"/>
+      <c r="C30" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>iDesign — школа практического дизайна</t>
@@ -2614,10 +2624,15 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="n"/>
+          <t>Отказ</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
       <c r="P30" t="n">
         <v>0</v>
       </c>
@@ -2625,7 +2640,7 @@
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr">
         <is>
-          <t>«Первая школа практического дизайна на Урале»; 200+ выпускников/год; 4 направления + детские/подростковые курсы; куратор Ольга Розет (БВШД); центр города (здание УрГАХА), 9–21 ежедневно; email отдела продаж именной || Соцсети: IG @i_design_school; ВК/TG заявлены в карточках, URL не найдены по сниппетам (не подтверждено)</t>
+          <t>«Первая школа практического дизайна на Урале»; 200+ выпускников/год; 4 направления + детские/подростковые курсы; куратор Ольга Розет (БВШД); центр города (здание УрГАХА), 9–21 ежедневно; email отдела продаж именной || Соцсети: IG @i_design_school; ВК/TG заявлены в карточках, URL не найдены по сниппетам (не подтверждено) || отправлено 07.07 04:18 UTC || ОТКАЗ 07.07: постоянный партнёр по продвижению. Больше не писать</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2651,9 @@
       <c r="B31" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C31" s="2" t="n"/>
+      <c r="C31" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>БьютиМед — клиника эстетической медицины</t>
@@ -2684,7 +2701,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N31" s="2" t="n"/>
@@ -2695,7 +2712,7 @@
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr">
         <is>
-          <t>2ГИС 4.9 (544!); ПроДокторов 17 врачей 283 отзыва; 30+ аппаратов, официальная площадка InMode; 2 локации (Советская 26а, Пермская 33); врачебная косметология — высокий чек; SEO развит, платные каналы недожаты || Соцсети: агрегатор указывает ВК/IG, ссылки не подтверждены по сниппетам</t>
+          <t>2ГИС 4.9 (544!); ПроДокторов 17 врачей 283 отзыва; 30+ аппаратов, официальная площадка InMode; 2 локации (Советская 26а, Пермская 33); врачебная косметология — высокий чек; SEO развит, платные каналы недожаты || Соцсети: агрегатор указывает ВК/IG, ссылки не подтверждены по сниппетам || отправлено 07.07 11:39 UTC</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2793,9 @@
       <c r="B33" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C33" s="2" t="n"/>
+      <c r="C33" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>МузКласс — школа современной музыки</t>
@@ -2824,7 +2843,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N33" s="2" t="n"/>
@@ -2835,7 +2854,7 @@
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Резерв: с 2016; вокал/гитара/барабаны/фортепиано/скрипка — много сегментов; 2 адреса в каталогах; конкурируют с федеральными сетями («Виртуозы», «Не Школа») || Соцсети: ВК vk.com/club113992055 (вероятно малоактивен); IG @muzclassnn; TG не найден || ПРОВЕРКА 07.07: школа жива, уже 3 адреса (расширение!); email актуален; актуальный ВК vk.com/muzclasscom; урок 60 мин — дифференциатор || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>Резерв: с 2016; вокал/гитара/барабаны/фортепиано/скрипка — много сегментов; 2 адреса в каталогах; конкурируют с федеральными сетями («Виртуозы», «Не Школа») || Соцсети: ВК vk.com/club113992055 (вероятно малоактивен); IG @muzclassnn; TG не найден || ПРОВЕРКА 07.07: школа жива, уже 3 адреса (расширение!); email актуален; актуальный ВК vk.com/muzclasscom; урок 60 мин — дифференциатор || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || отправлено 08.07 06:24 UTC — версия v1 (до HTML)</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2865,9 @@
       <c r="B34" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C34" s="2" t="n"/>
+      <c r="C34" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>Родная клиника — медцентр</t>
@@ -2894,7 +2915,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N34" s="2" t="n"/>
@@ -2905,7 +2926,7 @@
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Резерв: ПроДокторов 24 врача, 1570 отзывов; локомотив гинекология; раздел /landings/ на сайте — посадочные под платный трафик уже пробуют; одна точка на Ворошиловском || Соцсети: на сайте кнопки ВК/TG/WA, URL не подтверждены || ПРОВЕРКА 07.07: директор ПОДТВЕРЖДЁН — Родной Андрей Юрьевич (учредитель ООО «ЦДМ», checko); email актуален (ya.ru = алиас yandex.ru) || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>Резерв: ПроДокторов 24 врача, 1570 отзывов; локомотив гинекология; раздел /landings/ на сайте — посадочные под платный трафик уже пробуют; одна точка на Ворошиловском || Соцсети: на сайте кнопки ВК/TG/WA, URL не подтверждены || ПРОВЕРКА 07.07: директор ПОДТВЕРЖДЁН — Родной Андрей Юрьевич (учредитель ООО «ЦДМ», checko); email актуален (ya.ru = алиас yandex.ru) || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || отправлено 08.07 06:26 UTC — v1</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3476,7 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3487,9 @@
       <c r="B44" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C44" s="2" t="n"/>
+      <c r="C44" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>«Нимфа» — сеть салонов красоты (4 точки)</t>
@@ -3514,7 +3537,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N44" s="2" t="n"/>
@@ -3525,7 +3548,7 @@
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Сеть 4 салона; 4.6/140 2ГИС; премиум аппаратная+инъекционная косметология, лазерная эпиляция; ВЫДЕЛЕННЫЙ маркетинговый email (пишем на него); осн. ящик nimfa2002@bk.ru || Соцсети: IG @nimfa_omsk; ВК кнопка на картах, URL не подтверждён || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>Сеть 4 салона; 4.6/140 2ГИС; премиум аппаратная+инъекционная косметология, лазерная эпиляция; ВЫДЕЛЕННЫЙ маркетинговый email (пишем на него); осн. ящик nimfa2002@bk.ru || Соцсети: IG @nimfa_omsk; ВК кнопка на картах, URL не подтверждён || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || отправлено 08.07 06:49 UTC — v2 HTML</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3559,9 @@
       <c r="B45" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C45" s="2" t="n"/>
+      <c r="C45" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>SOHO — салон красоты и косметологии (3 филиала)</t>
@@ -3584,7 +3609,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N45" s="2" t="n"/>
@@ -3595,7 +3620,7 @@
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr">
         <is>
-          <t>С 2005, 26 сотрудников; 3 филиала вкл. ТЦ «Галерея Чижова»; отдельная косметологическая клиника (cosmetology-voronezh.ru, 6 врачей, 45 отзывов ПроДокторов) || Соцсети: ВК/TG упомянуты в 2ГИС, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>С 2005, 26 сотрудников; 3 филиала вкл. ТЦ «Галерея Чижова»; отдельная косметологическая клиника (cosmetology-voronezh.ru, 6 врачей, 45 отзывов ПроДокторов) || Соцсети: ВК/TG упомянуты в 2ГИС, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || отправлено 08.07 06:46 UTC — v2 HTML</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3690,7 @@
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
-          <t>2 филиала (Ястынская 7, Карамзина 13); Zoon 4.3; ученики занимаются 3–6 лет (высокий LTV); есть промо-лендинг promo.linguacity-school.ru — уже вкладываются в трафик || Соцсети: не найдены по сниппетам (не подтверждено) || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>2 филиала (Ястынская 7, Карамзина 13); Zoon 4.3; ученики занимаются 3–6 лет (высокий LTV); есть промо-лендинг promo.linguacity-school.ru — уже вкладываются в трафик || Соцсети: не найдены по сниппетам (не подтверждено) || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3771,9 @@
       <c r="B48" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C48" s="2" t="n"/>
+      <c r="C48" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D48" t="inlineStr">
         <is>
           <t>«Клиника в Северном» + «Первый частный травмпункт»</t>
@@ -3794,7 +3821,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N48" s="2" t="n"/>
@@ -3805,7 +3832,7 @@
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr">
         <is>
-          <t>56 врачей, 851 отзыв ПроДокторов; УНИКУМ: единственный в городе частный круглосуточный травмпункт — готовый оффер для Директа; агрегаторная зависимость (ПроДокторов/Фламп/Zoon/DocDoc) || Соцсети: ВК заявлен в orgpage, URL не подтверждён || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>56 врачей, 851 отзыв ПроДокторов; УНИКУМ: единственный в городе частный круглосуточный травмпункт — готовый оффер для Директа; агрегаторная зависимость (ПроДокторов/Фламп/Zoon/DocDoc) || Соцсети: ВК заявлен в orgpage, URL не подтверждён || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || отправлено 08.07 06:35 UTC — v1</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3843,9 @@
       <c r="B49" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C49" s="2" t="n"/>
+      <c r="C49" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>«Докториус» (экс-«Авиценна») — клиника</t>
@@ -3864,7 +3893,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N49" s="2" t="n"/>
@@ -3875,7 +3904,7 @@
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr">
         <is>
-          <t>ФАКТ-ЧЕК Яны 07.07: название «Докториус» используется минимум с 2023 (отзывы за май/сент/ноябрь 2023) — НЕ свежий ребрендинг, зацепка исправлена на «отзывная база + собственный канал»; 45 врачей, 1232 отзыва ПроДокторов; email ещё старый avicenna18@ || Соцсети: ВК vk.com/doktorius_klinica || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>ФАКТ-ЧЕК Яны 07.07: название «Докториус» используется минимум с 2023 (отзывы за май/сент/ноябрь 2023) — НЕ свежий ребрендинг, зацепка исправлена на «отзывная база + собственный канал»; 45 врачей, 1232 отзыва ПроДокторов; email ещё старый avicenna18@ || Соцсети: ВК vk.com/doktorius_klinica || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || отправлено 08.07 06:34 UTC — ЯНА ПЕРЕПИСАЛА САМА (тема «Заявки по фиксированной цене «Докториус»», ошибочный «ребрендинг» убран ею)</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4306,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -4297,7 +4326,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -4317,7 +4346,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -4327,7 +4356,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -4337,7 +4366,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.07407407407407407</v>
       </c>
     </row>
     <row r="11">
@@ -4387,7 +4416,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -4451,7 +4480,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -4476,7 +4505,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -4501,16 +4530,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.25</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -4570,16 +4599,16 @@
         </is>
       </c>
       <c r="B27" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
         <v>1</v>
       </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
       <c r="E27" s="4" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -4595,7 +4624,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -4604,7 +4633,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05263157894736842</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -4664,16 +4693,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.08</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -4689,7 +4718,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C33" t="n">
         <v>0</v>
@@ -4758,7 +4787,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C37" t="n">
         <v>0</v>
@@ -4767,7 +4796,7 @@
         <v>1</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>0.1</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -4783,16 +4812,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>0</v>
+        <v>0.0625</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -4905,28 +4934,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>0.0667</v>
+        <v>0.0741</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -5002,10 +5031,10 @@
         <v>53</v>
       </c>
       <c r="C2" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Micro letters v2: step-by-step ad mechanics, 2 critic agents feedback applied (budget benchmark, redo guarantee, no IG); followups D+3 recorded; batch-5 beauty/medicine dossiers in CRM
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S54"/>
+  <dimension ref="A1:S71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -632,7 +632,7 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Авторская клиника косметолога; лояльные клиенты 10+ лет; нет заметной рекламы в Директе/ВК, продвижение на сарафане</t>
+          <t>Авторская клиника косметолога; лояльные клиенты 10+ лет; нет заметной рекламы в Директе/ВК, продвижение на сарафане || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Два центра; врачебное позиционирование; активного ВК не видно — локальный таргет по Академгородку свободен</t>
+          <t>Два центра; врачебное позиционирование; активного ВК не видно — локальный таргет по Академгородку свободен || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Оффер «4 руки за 1,5 часа», гарантия на покрытие; запись только по телефону, нет онлайн-записи и промо-лендингов</t>
+          <t>Оффер «4 руки за 1,5 часа», гарантия на покрытие; запись только по телефону, нет онлайн-записи и промо-лендингов || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Программы «для двоих» и мужские SPA — сегменты под сертификаты; запись только по телефону, реклама сегментов не ведётся</t>
+          <t>Программы «для двоих» и мужские SPA — сегменты под сертификаты; запись только по телефону, реклама сегментов не ведётся || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Дети 6–17, занятия 1-на-1, своё приложение; дорогое привлечение, из соцсетей только устаревший Facebook</t>
+          <t>Дети 6–17, занятия 1-на-1, своё приложение; дорогое привлечение, из соцсетей только устаревший Facebook || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Академическая школа у метро Гражданский проспект, дети и взрослые, есть онлайн; сайт-визитка без воронки, живёт на сарафане</t>
+          <t>Академическая школа у метро Гражданский проспект, дети и взрослые, есть онлайн; сайт-визитка без воронки, живёт на сарафане || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Позиционирование «естественный результат, домашняя атмосфера»; активных соцсетей не видно — потенциал SMM + таргет ВК по Казани</t>
+          <t>Позиционирование «естественный результат, домашняя атмосфера»; активных соцсетей не видно — потенциал SMM + таргет ВК по Казани || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Рейтинг 4.7, 364 отзыва на 2ГИС, детский бренд «ДетиДент»; привлечение опирается на агрегаторы — точка роста Директ</t>
+          <t>Рейтинг 4.7, 364 отзыва на 2ГИС, детский бренд «ДетиДент»; привлечение опирается на агрегаторы — точка роста Директ || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>28 врачей, 936 отзывов на ПроДокторов; репутация на агрегаторах, собственный платный трафик недозагружен</t>
+          <t>28 врачей, 936 отзывов на ПроДокторов; репутация на агрегаторах, собственный платный трафик недозагружен || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
         </is>
       </c>
     </row>
@@ -3953,17 +3953,17 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ученики для «Ренессанс плюс» к осени</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N50" s="2" t="n"/>
@@ -4023,17 +4023,17 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Идея по записям для Uclinic</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N51" s="2" t="n"/>
@@ -4093,17 +4093,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Пациенты для филиалов «АртМеда»</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N52" s="2" t="n"/>
@@ -4163,17 +4163,17 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Пациенты для четырёх филиалов «Пересвета»</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
@@ -4255,6 +4255,1196 @@
       <c r="S54" t="inlineStr">
         <is>
           <t>Резерв на будущее (не дублировать Волгоград с Uclinic в одном батче)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>«Лоранж» — студия красоты</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Челябинск</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Салова Юлия Геннадьевна (директор ООО «Лоранж-ПРОФИ», с 2009)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>info@lorange.ru</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://www.lorange.ru/</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Идея по записям для «Лоранж»</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="n"/>
+      <c r="P55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="2" t="n"/>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>С 2003; 2ГИС 4.8 (285); «Лучший салон красоты 2023»; ~17 сотрудников; СПА/фитобочка/татуаж/инъекции; IG @lorange2003 1,7K; ВК заявлен, URL не подтверждён</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>«Океания» Clinic &amp; SPA</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Саратов</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Ермакова Екатерина Владимировна (директор ООО «Океания», с 2009)</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>info@salon-okeania.ru</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://okeanea.ru/</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Записи для двух филиалов «Океании»</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="n"/>
+      <c r="P56" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="2" t="n"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>2 филиала (косметология Рабочая 29/39, SPA Валовая 2/10); ПроДокторов 14 врачей 209 отзывов; без выходных 9–21; несколько сайтов — распылённый digital; ВК/TG заявлены, URL не подтверждены</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Институт красоты «Рашель»</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Ярославль</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Савельева Юлия Александровна (директор ООО «Салон Красоты «Рашель», с 2004)</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>administrator@rashele.ru</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://rashele.ru/</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Идея по записям для «Рашель»</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="n"/>
+      <c r="P57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="2" t="n"/>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>С 2004, особняк купца Ерыкалова XIX в. в центре (Кирова 12) — бренд-фактура; полный цикл; отзывы смешанные (Zoon/2ГИС) — угол «репутация+трафик»; соцсети не найдены по сниппетам (не подтверждено)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Языковая школа Дмитрия Никитина</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Ярославль</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Дмитрий Никитин (основатель, школа именная)</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>marketing.dnschool@gmail.com</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://dnschool.ru/</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Ученики для школы Никитина к сентябрю</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="n"/>
+      <c r="P58" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="2" t="n"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Яндекс «Хорошее место—2026», 4.9; 2ГИС 5.0; 3 локации; кембриджские экзамены; проекты для преподавателей; ЕСТЬ маркетинг-ящик; ВК vk.com/dnschoolclub; осн. email nikitindss@mail.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>LEO school — центр допобразования</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Иркутск</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>предположительно Шаравьёв В.А. (ООО «СОФОС» — ТРЕБУЕТ ПРОВЕРКИ, в письме без имени); сотрудник Ирина Краснюк</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>info@leo-irk.ru</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://leo-irk.ru/</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Набор к сентябрю для LEO school</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="n"/>
+      <c r="P59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="2" t="n"/>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>2 адреса + онлайн; 9 языков; летний интенсив ЕГЭ + лагерь; партнёр Liden&amp;Denz; РКИ, профориентация; ВК/TG не найдены по сниппетам (не подтверждено)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Стоматология «Эталон»</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Челябинск</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Нестерко Олег Александрович (гендиректор ООО «Эталон СК», с 2015; владелец Нестерко С.О.)</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>etalonclinic@mail.ru</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://etalonclinic.ru/</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Свои пациенты для «Эталона»</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="n"/>
+      <c r="P60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="2" t="n"/>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>2 филиала (Сони Кривой 38 центр, Марченко 16 ЧТЗ); ПроДокторов 71+50 отзывов; имплантология/ортодонтия/детская; ~21 чел.; ВК живой (vk сообщество etalonclinic74, бонусная механика); сайт заявляет 51 000+ пациентов. ПИСЬМО С ПРЕЗЕНТАЦИЕЙ (прикрепить вручную)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>«Имплант Люкс» — стоматология</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Саратов</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Аракелян Эдуард Зоревич (директор ООО «Имплант Люкс», он же ведущий ортопед; смены руководителя в истории — уточнить)</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>implantsar@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://implantsar.com/</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="n"/>
+      <c r="P61" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="2" t="n"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Резерв: ПроДокторов 11 врачей 137 отзывов, премии 2023/2024/2025; 2ГИС 4.9 (84); локомотив имплантация; с 2004; экс-главврач ушёл в 2025 — повод «перестройка маркетинга»</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>City Clinic — врачебная косметология</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Иркутск</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>cityclinic38@mail.ru</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://cityclinic38.ru/</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="n"/>
+      <c r="P62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="2" t="n"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Резерв: 2ГИС 4.5 (94); с 2016; лазер+инъекции+аппаратная; ЛПР не найден (минус для холодного захода); IG @cityclinic38; ВК/TG заявлены в 2ГИС</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Частная школа «Колибри»</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Челябинск</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>вероятно Майбородина Юлия Евгеньевна (директор связанного ЧДОУ — ТРЕБУЕТ ПРОВЕРКИ)</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>info@kolibri-school.ru</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://kolibri-school.ru/</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="n"/>
+      <c r="P63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" s="2" t="n"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Резерв: набор в 1–10 классы на 2026–27 (один источник — сверить); 3 здания + детсад (экосистема сад→школа); полный день 8–19, английский с носителями; соцсети не найдены по сниппетам</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>МассажТомск.рф — студия массажа</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Томск</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>massagvtomske@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://массажтомск.рф</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Новые клиенты для вашей студии — 18 000 ₽</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>price18</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="n"/>
+      <c r="P64" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q64" s="2" t="n"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Семейная студия с 2012; 4.9/120 на 2ГИС; ВК vk.com/MassagTomsk + TG подтверждены || Рекламная услуга для оффера: курс массажа спины</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>«Сахар Воск» — студия депиляции и массажа</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Киров</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Sv208300@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://сахар-воск.рф</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Новые клиенты для «Сахар Воск» — 18 000 ₽</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>price18</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="n"/>
+      <c r="P65" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" s="2" t="n"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Спасская 57; шугаринг жен/муж/подростки + массаж; ежедневно 10–21; ВК-группа подтверждена (Zoon) || Рекламная услуга для оффера: шугаринг бикини+ноги</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C66" s="2" t="n"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>«ШОК» — танцевальное пространство Ольги Козырьковой</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Калуга</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Ольга Козырькова (владелица, имя в названии)</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>shok.dance.kozyrkova@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://shok-dance-kaluga.ru/</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Новые ученики для «ШОК» — 18 000 ₽</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>price18</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="n"/>
+      <c r="P66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" s="2" t="n"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>С 2020; 2 площадки; зумба/high heels/танец живота/детская хореография; ВК не подтверждён — проверить || Рекламная услуга для оффера: набор детских групп хореографии (пробное)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>«Классика» — салон красоты</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Киров</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>klassika-pro@mail.ru</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://классикасалон.рф</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Новые клиенты для «Классики» — 18 000 ₽</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>price18</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="n"/>
+      <c r="P67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="2" t="n"/>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Ленина 79; 9–21; стрижки/ногти/брови/эпиляция/косметология; хвалят интерьер и персонал, отзывы смешанные; ВК/TG/WA подтверждены (Zoon) || Рекламная услуга для оффера: комплекс маникюр+педикюр</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>«Сахара» — студия шугаринга</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Рязань</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>sahararzn@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://sahararzn.ru/</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Новые клиенты для «Сахары» — 18 000 ₽</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>price18</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="n"/>
+      <c r="P68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="2" t="n"/>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>2 точки (БЦ Юпитер + Большая 102а); шугаринг/воск/лазер/SPA/ресницы-брови; ежедневно 10–21; ВК не подтверждён || Рекламная услуга для оффера: шугаринг для новых клиентов</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>LUNAMEL — салон красоты</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Тула</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>lunamel71@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://lunamel.clients.site/</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="n"/>
+      <c r="P69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="2" t="n"/>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Резерв micro: Советская 54Б, 10 лет; маникюр/педикюр/брови/ресницы; ВК не подтверждён || Рекламная услуга для оффера: маникюр с покрытием</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>«Вокальная Мастерская»</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Ульяновск</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ulvocal@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://vocal-ulyanovsk.ru/</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="n"/>
+      <c r="P70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="2" t="n"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Резерв micro: центр города; вокал/гитара/фортепиано; хвалят преподавателя Ирину; ВК не подтверждён || Рекламная услуга для оффера: уроки вокала для взрослых (бесплатное пробное)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>«Лизетта» — студия рисования</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Кемерово</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Елизавета Меднова (владелица, живописец-педагог)</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>lizettasite@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://lizetta.ru/</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="n"/>
+      <c r="P71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="2" t="n"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Резерв micro (на грани сегмента — 5 филиалов): первое занятие бесплатно || Рекламная услуга для оффера: курс рисования с нуля (первое бесплатно)</t>
         </is>
       </c>
     </row>
@@ -4296,7 +5486,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>53</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4">
@@ -4306,7 +5496,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -5028,7 +6218,7 @@
         <v>46209</v>
       </c>
       <c r="B2" t="n">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="C2" t="n">
         <v>27</v>

</xml_diff>

<commit_message>
Daily run 09.07: batch-1 followup reconciliation (6/9 sent by Yana 08.07), 10 followup drafts for batch-2 (send 10.07), Star Talk nudge draft pending approval, batch-6 assembled from existing drafts for 14.07 (pending-drafts cap alert), report rebuilt and republished
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S71"/>
+  <dimension ref="A1:S72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -626,13 +626,13 @@
       </c>
       <c r="N2" s="2" t="n"/>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Авторская клиника косметолога; лояльные клиенты 10+ лет; нет заметной рекламы в Директе/ВК, продвижение на сарафане || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
+          <t>Авторская клиника косметолога; лояльные клиенты 10+ лет; нет заметной рекламы в Директе/ВК, продвижение на сарафане || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — ОТПРАВЛЕН Яной 08.07; №2 — 15.07</t>
         </is>
       </c>
     </row>
@@ -698,13 +698,13 @@
       </c>
       <c r="N3" s="2" t="n"/>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Два центра; врачебное позиционирование; активного ВК не видно — локальный таргет по Академгородку свободен || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
+          <t>Два центра; врачебное позиционирование; активного ВК не видно — локальный таргет по Академгородку свободен || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — ОТПРАВЛЕН Яной 08.07; №2 — 15.07</t>
         </is>
       </c>
     </row>
@@ -770,13 +770,13 @@
       </c>
       <c r="N4" s="2" t="n"/>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" s="2" t="n"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Оффер «4 руки за 1,5 часа», гарантия на покрытие; запись только по телефону, нет онлайн-записи и промо-лендингов || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
+          <t>Оффер «4 руки за 1,5 часа», гарантия на покрытие; запись только по телефону, нет онлайн-записи и промо-лендингов || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — ОТПРАВЛЕН Яной 08.07; №2 — 15.07</t>
         </is>
       </c>
     </row>
@@ -842,13 +842,13 @@
       </c>
       <c r="N5" s="2" t="n"/>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5" s="2" t="n"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Программы «для двоих» и мужские SPA — сегменты под сертификаты; запись только по телефону, реклама сегментов не ведётся || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
+          <t>Программы «для двоих» и мужские SPA — сегменты под сертификаты; запись только по телефону, реклама сегментов не ведётся || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — ОТПРАВЛЕН Яной 08.07; №2 — 15.07</t>
         </is>
       </c>
     </row>
@@ -991,13 +991,13 @@
       </c>
       <c r="N7" s="2" t="n"/>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" s="2" t="n"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Дети 6–17, занятия 1-на-1, своё приложение; дорогое привлечение, из соцсетей только устаревший Facebook || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
+          <t>Дети 6–17, занятия 1-на-1, своё приложение; дорогое привлечение, из соцсетей только устаревший Facebook || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — ОТПРАВЛЕН Яной 08.07; №2 — 15.07</t>
         </is>
       </c>
     </row>
@@ -1279,13 +1279,13 @@
       </c>
       <c r="N11" s="2" t="n"/>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q11" s="2" t="n"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>28 врачей, 936 отзывов на ПроДокторов; репутация на агрегаторах, собственный платный трафик недозагружен || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — отправить 09.07</t>
+          <t>28 врачей, 936 отзывов на ПроДокторов; репутация на агрегаторах, собственный платный трафик недозагружен || Фоллоу-ап №1 (D+3) подготовлен 08.07 ответом в цепочку — ОТПРАВЛЕН Яной 08.07; №2 — 15.07</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Резерв: общий support-ящик и международный фокус — письмо на следующий день, если нужен добор квоты || ДОСЬЕ v2 (07.07): РФ-рынок активен (цены в рублях ~700–900₽/урок, 2ГИС Москва, свежие русские отзывы); основатель Сергей Жучков; партнёрство с МПГУ (Minecraft для учителей); привлекали $1,5M инвестиций; 20 000+ учеников; IG @progkids 21K; ВК упомянут в 2ГИС, URL не подтверждён</t>
+          <t>Резерв: общий support-ящик и международный фокус — письмо на следующий день, если нужен добор квоты || ДОСЬЕ v2 (07.07): РФ-рынок активен (цены в рублях ~700–900₽/урок, 2ГИС Москва, свежие русские отзывы); основатель Сергей Жучков; партнёрство с МПГУ (Minecraft для учителей); привлекали $1,5M инвестиций; 20 000+ учеников; IG @progkids 21K; ВК упомянут в 2ГИС, URL не подтверждён || Резерв батча №7</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Резерв: семейная многопрофильная клиника, слабее персонализация — дособрать факты перед письмом || ДОСЬЕ v2 (07.07): 30 врачей, 525 отзывов ПроДокторов, «Лучший медцентр 2023», номинант 2026; локомотивы: гинекология+УЗИ, педиатрия, эндокринология; НОВЫЙ филиал на Владимирской (5 отзывов — раскачать трафиком); ВК/TG не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:43 UTC</t>
+          <t>Резерв: семейная многопрофильная клиника, слабее персонализация — дособрать факты перед письмом || ДОСЬЕ v2 (07.07): 30 врачей, 525 отзывов ПроДокторов, «Лучший медцентр 2023», номинант 2026; локомотивы: гинекология+УЗИ, педиатрия, эндокринология; НОВЫЙ филиал на Владимирской (5 отзывов — раскачать трафиком); ВК/TG не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:43 UTC || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>16 лет, ТОП-клиник Сибири 2023; широкая линейка (лазер, вес, подология, трихология); брендовый спрос уходит агрегаторам || Соцсети: VK указан в контактах, но не находится в поиске; 2ГИС 4.7 (302 оценки); негатив — про администраторов || СОЦРАЗВЕДКА v2 (07.07, после ошибки): ВК ЕСТЬ — vk.com/altikansk (подтверждено Яной; сайт заявляет ВК/WhatsApp/TG, страница ВК не индексируется поиском). Письмо пересобрано: зацепка на репутации+ВК, утверждение об отсутствии убрано || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
+          <t>16 лет, ТОП-клиник Сибири 2023; широкая линейка (лазер, вес, подология, трихология); брендовый спрос уходит агрегаторам || Соцсети: VK указан в контактах, но не находится в поиске; 2ГИС 4.7 (302 оценки); негатив — про администраторов || СОЦРАЗВЕДКА v2 (07.07, после ошибки): ВК ЕСТЬ — vk.com/altikansk (подтверждено Яной; сайт заявляет ВК/WhatsApp/TG, страница ВК не индексируется поиском). Письмо пересобрано: зацепка на репутации+ВК, утверждение об отсутствии убрано || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>С 2017, аппаратная база InMode; раздел «Акции» на сайте — готовые офферы без трафика; врачи Эльвира Асхатовна, Ляйля Рамиловна || Соцсети: VK/TG не находятся; ПроДокторов 29 положительных отзывов || СОЦРАЗВЕДКА v2 (07.07): сайт заявляет ВК и Telegram (сниппеты контактов); IG @sovershenstvo_clinic. Письмо пересобрано: зацепка на разделе «Акции» без утверждений об отсутствии соцсетей || отправлено 07.07 02:35 UTC — НОВЫЙ черновик; Яна сама сменила тему на «Заявки для «Совершенства»»</t>
+          <t>С 2017, аппаратная база InMode; раздел «Акции» на сайте — готовые офферы без трафика; врачи Эльвира Асхатовна, Ляйля Рамиловна || Соцсети: VK/TG не находятся; ПроДокторов 29 положительных отзывов || СОЦРАЗВЕДКА v2 (07.07): сайт заявляет ВК и Telegram (сниппеты контактов); IG @sovershenstvo_clinic. Письмо пересобрано: зацепка на разделе «Акции» без утверждений об отсутствии соцсетей || отправлено 07.07 02:35 UTC — НОВЫЙ черновик; Яна сама сменила тему на «Заявки для «Совершенства»» || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
-          <t>19+ лет, 2 филиала (Восход 14/1, пл. К. Маркса); запись только по телефону; устаревший сайт без трафика || Соцсети: VK vk.com/terradelsol; Фламп/2ГИС 4.5 (~130 отзывов), хвалят косметолога Элеонору Винник и стилиста Татьяну Евдокимову || отправлено 07.07 02:44 UTC (корректный черновик от 06.07)</t>
+          <t>19+ лет, 2 филиала (Восход 14/1, пл. К. Маркса); запись только по телефону; устаревший сайт без трафика || Соцсети: VK vk.com/terradelsol; Фламп/2ГИС 4.5 (~130 отзывов), хвалят косметолога Элеонору Винник и стилиста Татьяну Евдокимову || отправлено 07.07 02:44 UTC (корректный черновик от 06.07) || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Полный комплекс услуг; личный gmail директора — короткий цикл сделки; нет онлайн-записи || Соцсети: VK/IG-ссылки на сайте, активного сообщества нет; Zoon/Фламп: хвалят стилиста Мане (Air Touch), мастеров Светлану и Виктора || СОЦРАЗВЕДКА v2 (07.07): yell.ru заявляет VK/IG; вероятный IG @krasivielyudi_official (принадлежность не подтверждена — тёзки в других городах). Письмо пересобрано: убрано «соцсети почти не живут», мягкая формулировка про карты/сарафан || отправлено 07.07 02:42 UTC — НОВЫЙ черновик (после соцразведки v2)</t>
+          <t>Полный комплекс услуг; личный gmail директора — короткий цикл сделки; нет онлайн-записи || Соцсети: VK/IG-ссылки на сайте, активного сообщества нет; Zoon/Фламп: хвалят стилиста Мане (Air Touch), мастеров Светлану и Виктора || СОЦРАЗВЕДКА v2 (07.07): yell.ru заявляет VK/IG; вероятный IG @krasivielyudi_official (принадлежность не подтверждена — тёзки в других городах). Письмо пересобрано: убрано «соцсети почти не живут», мягкая формулировка про карты/сарафан || отправлено 07.07 02:42 UTC — НОВЫЙ черновик (после соцразведки v2) || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3 || СОЦРАЗВЕДКА v2 (07.07): Telegram-канал ЕСТЬ — t.me/naydisebyamsk; IG @naydisebya_ru 8,2K + @naydisebya.online; ВК не найден по сниппетам (не подтверждено). Письмо пересобрано: TG признан активом, утверждение «TG не развит» убрано || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
+          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3 || СОЦРАЗВЕДКА v2 (07.07): Telegram-канал ЕСТЬ — t.me/naydisebyamsk; IG @naydisebya_ru 8,2K + @naydisebya.online; ВК не найден по сниппетам (не подтверждено). Письмо пересобрано: TG признан активом, утверждение «TG не развит» убрано || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>IELTS/TOEFL/ЕГЭ + дети 4–12; сезонное окно — набор к учебному году; конкуренты (Skyeng) активно закупают трафик || Соцсети: VK/TG не видны в поиске; 20 отзывов на Kurshub (хвалят цену и расписание); Zoon, 2ГИС || СОЦРАЗВЕДКА v2 (07.07): сайт на странице контактов заявляет YouTube и ВКонтакте; TG — только бот-лидмагнит. Письмо пересобрано: «на сайте заявлены YouTube и ВК», без утверждений об отсутствии || отправлено 07.07 02:37 UTC — УШЛА СТАРАЯ ВЕРСИЯ (формулировка «ВК и TG в поиске почти не видны» — мягкая, риск низкий; сайт ВК заявляет). Новый неотправленный черновик r-1267307485728993365 УДАЛИТЬ. Если ответят про ВК — признать и перевести в пользу: «поэтому и пишем — аудиторию надо развивать рекламой»</t>
+          <t>IELTS/TOEFL/ЕГЭ + дети 4–12; сезонное окно — набор к учебному году; конкуренты (Skyeng) активно закупают трафик || Соцсети: VK/TG не видны в поиске; 20 отзывов на Kurshub (хвалят цену и расписание); Zoon, 2ГИС || СОЦРАЗВЕДКА v2 (07.07): сайт на странице контактов заявляет YouTube и ВКонтакте; TG — только бот-лидмагнит. Письмо пересобрано: «на сайте заявлены YouTube и ВК», без утверждений об отсутствии || отправлено 07.07 02:37 UTC — УШЛА СТАРАЯ ВЕРСИЯ (формулировка «ВК и TG в поиске почти не видны» — мягкая, риск низкий; сайт ВК заявляет). Новый неотправленный черновик r-1267307485728993365 УДАЛИТЬ. Если ответят про ВК — признать и перевести в пользу: «поэтому и пишем — аудиторию надо развивать рекламой» || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1925,7 @@
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Огромная контентная база и лид-магниты (выкройки, вебинары) без платного трафика; офлайн Мск+СПб + онлайн — идеальный матч под кейс Кинезио || Соцсети: Личный бренд Марии в IG @mari_amochaeva (заблокирован); YouTube + Rutube 514 подборок; VK/TG школы не видны; блог на сайте заброшен (статья 2020 г.) || СОЦРАЗВЕДКА v2 (07.07): ВК — целая живая сеть: vk.com/wanttosew (блог), vk.com/i_want_to_sew_spb, vk.com/wanttosew_msk + vkvideo.ru/@wanttosew; IG @wanttosew ~180K. Письмо пересобрано полностью: сообщества ВК = готовая воронка, оффер — направить на них платный трафик || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
+          <t>Огромная контентная база и лид-магниты (выкройки, вебинары) без платного трафика; офлайн Мск+СПб + онлайн — идеальный матч под кейс Кинезио || Соцсети: Личный бренд Марии в IG @mari_amochaeva (заблокирован); YouTube + Rutube 514 подборок; VK/TG школы не видны; блог на сайте заброшен (статья 2020 г.) || СОЦРАЗВЕДКА v2 (07.07): ВК — целая живая сеть: vk.com/wanttosew (блог), vk.com/i_want_to_sew_spb, vk.com/wanttosew_msk + vkvideo.ru/@wanttosew; IG @wanttosew ~180K. Письмо пересобрано полностью: сообщества ВК = готовая воронка, оффер — направить на них платный трафик || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Премиум: БЦ Corner Place, врачи из моск. института пластической хирургии, чек до 56 200 ₽ — юнит-экономика Директа сходится с запасом || Соцсети: VK/TG/IG не находятся; ПроДокторов 170 отзывов, 18 врачей || СОЦРАЗВЕДКА v2 (07.07): IG ЕСТЬ — @lancette_nn; ВК не найден (безопасно, но не утверждаем); TG — упоминание в 2ГИС без ссылки. Письмо пересобрано: IG признан активом, «нет ни ВК ни TG» убрано</t>
+          <t>Премиум: БЦ Corner Place, врачи из моск. института пластической хирургии, чек до 56 200 ₽ — юнит-экономика Директа сходится с запасом || Соцсети: VK/TG/IG не находятся; ПроДокторов 170 отзывов, 18 врачей || СОЦРАЗВЕДКА v2 (07.07): IG ЕСТЬ — @lancette_nn; ВК не найден (безопасно, но не утверждаем); TG — упоминание в 2ГИС без ссылки. Письмо пересобрано: IG признан активом, «нет ни ВК ни TG» убрано || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис) || СОЦРАЗВЕДКА v2 (07.07): соцсети этой клиники не найдены, НО в Екб есть стоматология-ТЁЗКА «Визави» (centrvizavi.ru, Шейнкмана 9) с ВК/TG — риск перепутать. Письмо пересобрано: «судя по открытым данным» вместо категоричного «канала нет» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v3 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r-5266668500978660320 удалить || отправлено 07.07 04:50 UTC — v3 с презентацией</t>
+          <t>14 специалистов, стаж ~23 года, приём 8–21; два параллельных сайта — несистемный маркетинг; полная зависимость от агрегаторов. dental=true || Соцсети: VK/TG отсутствуют; ПроДокторов 38 отзывов; 32top 4.7 vs Zoon 3.8 (негатив про сервис) || СОЦРАЗВЕДКА v2 (07.07): соцсети этой клиники не найдены, НО в Екб есть стоматология-ТЁЗКА «Визави» (centrvizavi.ru, Шейнкмана 9) с ВК/TG — риск перепутать. Письмо пересобрано: «судя по открытым данным» вместо категоричного «канала нет» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v3 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r-5266668500978660320 удалить || отправлено 07.07 04:50 UTC — v3 с презентацией || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2139,7 @@
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: ВК/TG не видны (Facebook в разведке не учитываем); Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258) || СОЦРАЗВЕДКА v2 (07.07): ВК/TG/IG не найдены ни на сайте, ни поиском (самый чистый кейс), но по правилу «не утверждать отсутствие» формулировка смягчена: «если запись идёт в основном с карт…». Есть заброшенный FB (игнорируем) || отправлено 07.07 01:55 UTC — НОВЫЙ черновик (v3); Яна сама сменила тему на «Заявки для стоматологий с фиксированной ценой» || ПРЕЗЕНТАЦИЯ: холодное письмо ушло 07.07 без вложения — приложить «OMG-кейсы-стоматологии.pptx» к фоллоу-апу D+3 (10.07), это сильный повод для второго касания</t>
+          <t>Маржинальные направления: имплантация, хирургия, микроскоп; репутация конвертируется только через карты. dental=true || Соцсети: ВК/TG не видны (Facebook в разведке не учитываем); Яндекс 4.8 (~4 865 оценок), 2ГИС 4.9 (258) || СОЦРАЗВЕДКА v2 (07.07): ВК/TG/IG не найдены ни на сайте, ни поиском (самый чистый кейс), но по правилу «не утверждать отсутствие» формулировка смягчена: «если запись идёт в основном с карт…». Есть заброшенный FB (игнорируем) || отправлено 07.07 01:55 UTC — НОВЫЙ черновик (v3); Яна сама сменила тему на «Заявки для стоматологий с фиксированной ценой» || ПРЕЗЕНТАЦИЯ: холодное письмо ушло 07.07 без вложения — приложить «OMG-кейсы-стоматологии.pptx» к фоллоу-апу D+3 (10.07), это сильный повод для второго касания || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Резерв: рейтинг ниже конкурентов, нет ЛПР; anti-age авторские методики — фактура для креативов || Соцсети: IG @timeless_studio_massage основной канал; VK не найден; Zoon 3.4; 2 филиала || ДОСЬЕ v2 (07.07): email info@timeless-studio.ru подтверждён в сниппетах сайта; сооснователи найдены; сайт делало агентство Chipsa (WebGL) — в упаковку вложились; 3 вакансии на hh — расширяются; открыты 07.2020, Петроградка, 9–22; 2ГИС показывает кнопку ВК (URL не подтверждён)</t>
+          <t>Резерв: рейтинг ниже конкурентов, нет ЛПР; anti-age авторские методики — фактура для креативов || Соцсети: IG @timeless_studio_massage основной канал; VK не найден; Zoon 3.4; 2 филиала || ДОСЬЕ v2 (07.07): email info@timeless-studio.ru подтверждён в сниппетах сайта; сооснователи найдены; сайт делало агентство Chipsa (WebGL) — в упаковку вложились; 3 вакансии на hh — расширяются; открыты 07.2020, Петроградка, 9–22; 2ГИС показывает кнопку ВК (URL не подтверждён) || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата || ДОСЬЕ v2 (07.07): ВК НАЙДЕН — vk.com/triars_school (сниппет Яндекс.Карт); также IG @triars_school, YouTube, Pinterest, TG как канал связи; с 2017; ЛПР не найден (вход через препода Марата); вакансии на hh (employer/3265114) — растут; платной рекламы не видно || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
+          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата || ДОСЬЕ v2 (07.07): ВК НАЙДЕН — vk.com/triars_school (сниппет Яндекс.Карт); также IG @triars_school, YouTube, Pinterest, TG как канал связи; с 2017; ЛПР не найден (вход через препода Марата); вакансии на hh (employer/3265114) — растут; платной рекламы не видно || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || Резерв батча №7</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1 || ДОСЬЕ v2 (07.07): ООО «Стоматология XXI век» (ИНН 1660130086, с 2009); акционные лендинги на сайте («кариес 5900₽») — готовы к трафику; ВК/TG не найдены по сниппетам (не подтверждено); одна точка — ЖК «Казань XXI век» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v2 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r5373719259897128450 удалить</t>
+          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1 || ДОСЬЕ v2 (07.07): ООО «Стоматология XXI век» (ИНН 1660130086, с 2009); акционные лендинги на сайте («кариес 5900₽») — готовы к трафику; ВК/TG не найдены по сниппетам (не подтверждено); одна точка — ЖК «Казань XXI век» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v2 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r5373719259897128450 удалить || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Yell 5.0 (18), ПроДокторов 48 врачей ~500 отзывов; в отзывах хвалят LPG и Fotona (пигментация за 2 сеанса); с 2018, 7 дней/нед; верх ICP по размеру || Соцсети: IG @laplas_clinic; ВК/TG не найдены по сниппетам (не подтверждено); живут на агрегаторах и картах || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
+          <t>Yell 5.0 (18), ПроДокторов 48 врачей ~500 отзывов; в отзывах хвалят LPG и Fotona (пигментация за 2 сеанса); с 2018, 7 дней/нед; верх ICP по размеру || Соцсети: IG @laplas_clinic; ВК/TG не найдены по сниппетам (не подтверждено); живут на агрегаторах и картах || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
-          <t>2ГИС 4.9 (69); MeDioStar NeXT Pro + Asclepion Dermablate; 3 филиала (Краснодар/Туапсе/Новороссийск); онлайн-запись YClients; эстетическая гинекология — маржинальная услуга; ЛПР не найден — уточнить на созвоне || Соцсети: IG laser_house23; ВК/TG не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:39 UTC</t>
+          <t>2ГИС 4.9 (69); MeDioStar NeXT Pro + Asclepion Dermablate; 3 филиала (Краснодар/Туапсе/Новороссийск); онлайн-запись YClients; эстетическая гинекология — маржинальная услуга; ЛПР не найден — уточнить на созвоне || Соцсети: IG laser_house23; ВК/TG не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:39 UTC || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2563,7 @@
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Яндекс 5.0 при 574 отзывах; «салон в стиле Бали» с бесплатным баром, dog-friendly; акция маникюр+гель-лак 2190₽ — промо уже используют; личный gmail на сайте — короткий цикл сделки || Соцсети: не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:41 UTC (старый CTA-A — уже в поле)</t>
+          <t>Яндекс 5.0 при 574 отзывах; «салон в стиле Бали» с бесплатным баром, dog-friendly; акция маникюр+гель-лак 2190₽ — промо уже используют; личный gmail на сайте — короткий цикл сделки || Соцсети: не найдены по сниппетам (не подтверждено) || отправлено 07.07 11:41 UTC (старый CTA-A — уже в поле) || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr">
         <is>
-          <t>2ГИС 4.9 (544!); ПроДокторов 17 врачей 283 отзыва; 30+ аппаратов, официальная площадка InMode; 2 локации (Советская 26а, Пермская 33); врачебная косметология — высокий чек; SEO развит, платные каналы недожаты || Соцсети: агрегатор указывает ВК/IG, ссылки не подтверждены по сниппетам || отправлено 07.07 11:39 UTC</t>
+          <t>2ГИС 4.9 (544!); ПроДокторов 17 врачей 283 отзыва; 30+ аппаратов, официальная площадка InMode; 2 локации (Советская 26а, Пермская 33); врачебная косметология — высокий чек; SEO развит, платные каналы недожаты || Соцсети: агрегатор указывает ВК/IG, ссылки не подтверждены по сниппетам || отправлено 07.07 11:39 UTC || Фоллоу-ап №1 (D+3) подготовлен 09.07 — отправить 10.07</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Резерв (верхняя граница ICP — крупный): Яндекс 4.8 (227); 3 этажа, 1500+ услуг, 2 адреса; активны на скидочных агрегаторах (СКИДКОМ, Lovefit) — платят за лидов, аргумент пересадить бюджет на ВК/Директ || Соцсети: 2ГИС показывает кнопки ВК/WA/TG, URL не подтверждены || ПРОВЕРКА 07.07: email подтверждён (+ запасной team@giovane-clinic.ru); 2ГИС 4.6/442; ПроДокторов 25 врачей; APTOS-сертификация || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>Резерв (верхняя граница ICP — крупный): Яндекс 4.8 (227); 3 этажа, 1500+ услуг, 2 адреса; активны на скидочных агрегаторах (СКИДКОМ, Lovefit) — платят за лидов, аргумент пересадить бюджет на ВК/Директ || Соцсети: 2ГИС показывает кнопки ВК/WA/TG, URL не подтверждены || ПРОВЕРКА 07.07: email подтверждён (+ запасной team@giovane-clinic.ru); 2ГИС 4.6/442; ПроДокторов 25 врачей; APTOS-сертификация || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
+          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || Резерв батча №7</t>
         </is>
       </c>
     </row>
@@ -3690,7 +3690,7 @@
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
-          <t>2 филиала (Ястынская 7, Карамзина 13); Zoon 4.3; ученики занимаются 3–6 лет (высокий LTV); есть промо-лендинг promo.linguacity-school.ru — уже вкладываются в трафик || Соцсети: не найдены по сниппетам (не подтверждено) || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить</t>
+          <t>2 филиала (Ястынская 7, Карамзина 13); Zoon 4.3; ученики занимаются 3–6 лет (высокий LTV); есть промо-лендинг promo.linguacity-school.ru — уже вкладываются в трафик || Соцсети: не найдены по сниппетам (не подтверждено) || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
-          <t>С 1998, лицензированная; 3 локации; IELTS/TOEFL/FCE + ЕГЭ/ОГЭ + обучение за рубежом (высокий чек); рейтинг лучших школ города (1tmn.ru) || Соцсети: ВК vk.com/livinglanguage (подтверждён), IG @living_language; TG не найден || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить</t>
+          <t>С 1998, лицензированная; 3 локации; IELTS/TOEFL/FCE + ЕГЭ/ОГЭ + обучение за рубежом (высокий чек); рейтинг лучших школ города (1tmn.ru) || Соцсети: ВК vk.com/livinglanguage (подтверждён), IG @living_language; TG не найден || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || БАТЧ №6: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -4954,7 +4954,7 @@
       <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr">
         <is>
-          <t>Семейная студия с 2012; 4.9/120 на 2ГИС; ВК vk.com/MassagTomsk + TG подтверждены || Рекламная услуга для оффера: курс массажа спины</t>
+          <t>Семейная студия с 2012; 4.9/120 на 2ГИС; ВК vk.com/MassagTomsk + TG подтверждены || Рекламная услуга для оффера: курс массажа спины || v2 (08.07, по указанию Яны + 2 агента-критика): пошаговая механика рекламы, ориентир бюджета «от 500 ₽/день, деньги идут ВКонтакте, не нам», гарантия «не напишет никто за неделю — переделаем бесплатно», убраны «под ключ»/«Media Group» из первой строки/Instagram-ссылка; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr">
         <is>
-          <t>Спасская 57; шугаринг жен/муж/подростки + массаж; ежедневно 10–21; ВК-группа подтверждена (Zoon) || Рекламная услуга для оффера: шугаринг бикини+ноги</t>
+          <t>Спасская 57; шугаринг жен/муж/подростки + массаж; ежедневно 10–21; ВК-группа подтверждена (Zoon) || Рекламная услуга для оффера: шугаринг бикини+ноги || v2 (08.07, по указанию Яны + 2 агента-критика): пошаговая механика рекламы, ориентир бюджета «от 500 ₽/день, деньги идут ВКонтакте, не нам», гарантия «не напишет никто за неделю — переделаем бесплатно», убраны «под ключ»/«Media Group» из первой строки/Instagram-ссылка; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5094,7 @@
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr">
         <is>
-          <t>С 2020; 2 площадки; зумба/high heels/танец живота/детская хореография; ВК не подтверждён — проверить || Рекламная услуга для оффера: набор детских групп хореографии (пробное)</t>
+          <t>С 2020; 2 площадки; зумба/high heels/танец живота/детская хореография; ВК не подтверждён — проверить || Рекламная услуга для оффера: набор детских групп хореографии (пробное) || v2 (08.07, по указанию Яны + 2 агента-критика): пошаговая механика рекламы, ориентир бюджета «от 500 ₽/день, деньги идут ВКонтакте, не нам», гарантия «не напишет никто за неделю — переделаем бесплатно», убраны «под ключ»/«Media Group» из первой строки/Instagram-ссылка; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -5164,7 +5164,7 @@
       <c r="R67" t="inlineStr"/>
       <c r="S67" t="inlineStr">
         <is>
-          <t>Ленина 79; 9–21; стрижки/ногти/брови/эпиляция/косметология; хвалят интерьер и персонал, отзывы смешанные; ВК/TG/WA подтверждены (Zoon) || Рекламная услуга для оффера: комплекс маникюр+педикюр</t>
+          <t>Ленина 79; 9–21; стрижки/ногти/брови/эпиляция/косметология; хвалят интерьер и персонал, отзывы смешанные; ВК/TG/WA подтверждены (Zoon) || Рекламная услуга для оффера: комплекс маникюр+педикюр || v2 (08.07, по указанию Яны + 2 агента-критика): пошаговая механика рекламы, ориентир бюджета «от 500 ₽/день, деньги идут ВКонтакте, не нам», гарантия «не напишет никто за неделю — переделаем бесплатно», убраны «под ключ»/«Media Group» из первой строки/Instagram-ссылка; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr">
         <is>
-          <t>2 точки (БЦ Юпитер + Большая 102а); шугаринг/воск/лазер/SPA/ресницы-брови; ежедневно 10–21; ВК не подтверждён || Рекламная услуга для оффера: шугаринг для новых клиентов</t>
+          <t>2 точки (БЦ Юпитер + Большая 102а); шугаринг/воск/лазер/SPA/ресницы-брови; ежедневно 10–21; ВК не подтверждён || Рекламная услуга для оффера: шугаринг для новых клиентов || v2 (08.07, по указанию Яны + 2 агента-критика): пошаговая механика рекламы, ориентир бюджета «от 500 ₽/день, деньги идут ВКонтакте, не нам», гарантия «не напишет никто за неделю — переделаем бесплатно», убраны «под ключ»/«Media Group» из первой строки/Instagram-ссылка; старый черновик удалить</t>
         </is>
       </c>
     </row>
@@ -5445,6 +5445,76 @@
       <c r="S71" t="inlineStr">
         <is>
           <t>Резерв micro (на грани сегмента — 5 филиалов): первое занятие бесплатно || Рекламная услуга для оффера: курс рисования с нуля (первое бесплатно)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C72" s="2" t="n"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>«Интер-Лэнг» — сеть школ иностранных языков</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Ярославль</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Передреева Анна Вячеславовна (директор ЧУ ДО, с 2007)</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>inter-lang_yar@mail.ru</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://www.inter-lang.ru/</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>Резерв</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="n"/>
+      <c r="P72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="2" t="n"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Резерв (сильный, 5/5): 5+ филиалов по районам (2ГИС подтверждает) — идеально под геотаргет; 3000+ учеников/год; линейка: английский/китайский/ментальная арифметика/скорочтение — сегментация кампаний; ВК/TG заявлены, URL не подтверждены</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5556,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -5506,7 +5576,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -6218,7 +6288,7 @@
         <v>46209</v>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C2" t="n">
         <v>27</v>

</xml_diff>

<commit_message>
Letters v4 for all 20 unsent leads: PDF case decks (funnel-to-revenue), work mechanics (sole-prop billing, own ad accounts, 1-2 payments/mo, KPI after test week, free lead-handling QA), one-word mediaplan CTA; reconcile 8 unrecorded sends + 3 followups sent by Yana; diff-review step added to playbook
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -1334,7 +1334,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Родители для ProgKids из Директа</t>
+          <t>Заявки ×2,5: медиаплан для ProgKids</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1355,7 +1355,7 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Резерв: общий support-ящик и международный фокус — письмо на следующий день, если нужен добор квоты || ДОСЬЕ v2 (07.07): РФ-рынок активен (цены в рублях ~700–900₽/урок, 2ГИС Москва, свежие русские отзывы); основатель Сергей Жучков; партнёрство с МПГУ (Minecraft для учителей); привлекали $1,5M инвестиций; 20 000+ учеников; IG @progkids 21K; ВК упомянут в 2ГИС, URL не подтверждён || Резерв батча №7</t>
+          <t>Резерв: общий support-ящик и международный фокус — письмо на следующий день, если нужен добор квоты || ДОСЬЕ v2 (07.07): РФ-рынок активен (цены в рублях ~700–900₽/урок, 2ГИС Москва, свежие русские отзывы); основатель Сергей Жучков; партнёрство с МПГУ (Minecraft для учителей); привлекали $1,5M инвестиций; 20 000+ учеников; IG @progkids 21K; ВК упомянут в 2ГИС, URL не подтверждён || Резерв батча №7 || БАТЧ №6 (v4): отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="2" t="n"/>
       <c r="R13" t="inlineStr"/>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Идея по записям для «Алтики»</t>
+          <t>Рост с 33 до 191 заявки в месяц: медиаплан для «Алтики»</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1724,7 +1724,9 @@
       <c r="B18" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C18" s="2" t="n"/>
+      <c r="C18" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>Школа рисования «Найди Себя»</t>
@@ -1772,7 +1774,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N18" s="2" t="n"/>
@@ -1783,7 +1785,7 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3 || СОЦРАЗВЕДКА v2 (07.07): Telegram-канал ЕСТЬ — t.me/naydisebyamsk; IG @naydisebya_ru 8,2K + @naydisebya.online; ВК не найден по сниппетам (не подтверждено). Письмо пересобрано: TG признан активом, утверждение «TG не развит» убрано || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || БАТЧ №6: отправка вт 14.07</t>
+          <t>С 2011; онлайн-курсы 990–2 500 ₽ — низкий чек, нужны дешёвые лиды; YouTube есть || Соцсети: IG @naydisebya_ru ~8 200 подписчиков (заблокирован в РФ); VK/TG не развиты; Zoon 4.3 || СОЦРАЗВЕДКА v2 (07.07): Telegram-канал ЕСТЬ — t.me/naydisebyamsk; IG @naydisebya_ru 8,2K + @naydisebya.online; ВК не найден по сниппетам (не подтверждено). Письмо пересобрано: TG признан активом, утверждение «TG не развит» убрано || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || ОТПРАВЛЕНО 08.07 (сверка 09.07)</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1906,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Идея для «Хочу Шить» к осеннему набору</t>
+          <t>Заявки ×2,5 к осеннему набору: медиаплан для «Хочу Шить»</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1974,7 +1976,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Пациентки для «Ланцета» — не только с ПроДокторов</t>
+          <t>1,14 млн ₽ с таргета за месяц: медиаплан для «Ланцета»</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2188,7 +2190,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Идея по записям для Timeless</t>
+          <t>44 465 заявок на массаж: медиаплан для Timeless</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2258,7 +2260,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Идея для «Триарс» к осеннему набору</t>
+          <t>Ученики к осеннему набору: медиаплан для «Триарс»</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2279,7 +2281,7 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата || ДОСЬЕ v2 (07.07): ВК НАЙДЕН — vk.com/triars_school (сниппет Яндекс.Карт); также IG @triars_school, YouTube, Pinterest, TG как канал связи; с 2017; ЛПР не найден (вход через препода Марата); вакансии на hh (employer/3265114) — растут; платной рекламы не видно || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || Резерв батча №7</t>
+          <t>Резерв: 2 адреса + онлайн, курс цифровой графики; дубль ниши с «Найди Себя» в батче 07.07 || Соцсети: VK-иконка на сайте, сообщество не индексируется; FB заблокирован; Фламп/2ГИС хвалят преподавателя Марата || ДОСЬЕ v2 (07.07): ВК НАЙДЕН — vk.com/triars_school (сниппет Яндекс.Карт); также IG @triars_school, YouTube, Pinterest, TG как канал связи; с 2017; ЛПР не найден (вход через препода Марата); вакансии на hh (employer/3265114) — растут; платной рекламы не видно || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || Резерв батча №7 || БАТЧ №6 (v4): отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2292,9 @@
       <c r="B26" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="C26" s="2" t="n"/>
+      <c r="C26" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>Стоматология «21 Век»</t>
@@ -2338,7 +2342,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N26" s="2" t="n"/>
@@ -2349,7 +2353,7 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1 || ДОСЬЕ v2 (07.07): ООО «Стоматология XXI век» (ИНН 1660130086, с 2009); акционные лендинги на сайте («кариес 5900₽») — готовы к трафику; ВК/TG не найдены по сниппетам (не подтверждено); одна точка — ЖК «Казань XXI век» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v2 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r5373719259897128450 удалить || БАТЧ №6: отправка вт 14.07</t>
+          <t>Резерв: семейная с детским приёмом (сегмент «мамы»), рассрочка — оффер для Директа; 3-я стоматология в батче — отложена || Соцсети: VK/TG отсутствуют; ПроДокторов 163 отзыва (~4.25), Zoon 4.1 || ДОСЬЕ v2 (07.07): ООО «Стоматология XXI век» (ИНН 1660130086, с 2009); акционные лендинги на сайте («кариес 5900₽») — готовы к трафику; ВК/TG не найдены по сниппетам (не подтверждено); одна точка — ЖК «Казань XXI век» || ПРЕЗЕНТАЦИЯ (07.07): письмо пересобрано v2 — добавлена строка о вложении «OMG-кейсы-стоматологии.pptx»; файл прикрепляет Яна вручную перед отправкой. Старый черновик r5373719259897128450 удалить || ОТПРАВЛЕНО 07.07 (сверка 09.07)</t>
         </is>
       </c>
     </row>
@@ -2398,7 +2402,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Идея по записям для LAPLAS</t>
+          <t>LPG-заявки по 475 ₽: медиаплан для LAPLAS</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2557,7 +2561,7 @@
       </c>
       <c r="N29" s="2" t="n"/>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q29" s="2" t="n"/>
       <c r="R29" t="inlineStr"/>
@@ -2706,7 +2710,7 @@
       </c>
       <c r="N31" s="2" t="n"/>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q31" s="2" t="n"/>
       <c r="R31" t="inlineStr"/>
@@ -2761,7 +2765,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Идея по записям для Giovane</t>
+          <t>Заявки по 488 ₽ вместо комиссий агрегаторам: медиаплан для Giovane</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3417,7 +3421,9 @@
       <c r="B43" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C43" s="2" t="n"/>
+      <c r="C43" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Face &amp; Body — клиника косметологии и гинекологии</t>
@@ -3465,7 +3471,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N43" s="2" t="n"/>
@@ -3476,7 +3482,7 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || Резерв батча №7</t>
+          <t>Лауреат Национальной премии по косметологии (2011); 11 врачей, 118 отзывов ПроДокторов; под тем же юрлицом (ООО «Медиас») центр эпиляции Epicenter; ЛПР противоречив (Верещагина И.С. либо Медведев А.Ю.) — в письме без имени || Соцсети: ВК/ОК/IG упомянуты на контактах, URL не подтверждены || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || CTA-v3 (08.07): запретная фраза «Ответьте „да“…без обязательств» заменена на «Прислать? Ответьте на это письмо…»; формат HTML с гиперссылками; отправлять самый свежий черновик, ранние удалить || ОТПРАВЛЕНО 08.07 (сверка 09.07)</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3675,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Ученики для Lingua City к сентябрю</t>
+          <t>Ученики к сентябрю: медиаплан для Lingua City</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3701,7 +3707,9 @@
       <c r="B47" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C47" s="2" t="n"/>
+      <c r="C47" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>«Живой Язык» — языковая школа</t>
@@ -3749,7 +3757,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N47" s="2" t="n"/>
@@ -3760,7 +3768,7 @@
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
-          <t>С 1998, лицензированная; 3 локации; IELTS/TOEFL/FCE + ЕГЭ/ОГЭ + обучение за рубежом (высокий чек); рейтинг лучших школ города (1tmn.ru) || Соцсети: ВК vk.com/livinglanguage (подтверждён), IG @living_language; TG не найден || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || БАТЧ №6: отправка вт 14.07</t>
+          <t>С 1998, лицензированная; 3 локации; IELTS/TOEFL/FCE + ЕГЭ/ОГЭ + обучение за рубежом (высокий чек); рейтинг лучших школ города (1tmn.ru) || Соцсети: ВК vk.com/livinglanguage (подтверждён), IG @living_language; TG не найден || v2 (07.07): HTML-версия с гиперссылками (сайт+TG+IG), вычитка текста; старый черновик удалить || ОТПРАВЛЕНО 08.07 (сверка 09.07)</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3923,9 @@
       <c r="B50" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C50" s="2" t="n"/>
+      <c r="C50" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D50" t="inlineStr">
         <is>
           <t>«Ренессанс плюс» — частная школа искусств</t>
@@ -3963,7 +3973,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N50" s="2" t="n"/>
@@ -3974,7 +3984,7 @@
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Резерв: с 2012, 1400+ учеников, 12 направлений (вокал/инструменты/живопись/актёрское); взрослые И дети 5+; концерты — готовый контент; слабое соцприсутствие</t>
+          <t>Резерв: с 2012, 1400+ учеников, 12 направлений (вокал/инструменты/живопись/актёрское); взрослые И дети 5+; концерты — готовый контент; слабое соцприсутствие || ОТПРАВЛЕНО 08.07 (сверка 09.07)</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4033,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Идея по записям для Uclinic</t>
+          <t>Окупаемость ×3,3: медиаплан для Uclinic</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -4093,7 +4103,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Пациенты для филиалов «АртМеда»</t>
+          <t>Выручка ×1,6 при бюджете −43%: медиаплан для «АртМеда»</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4125,7 +4135,9 @@
       <c r="B53" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C53" s="2" t="n"/>
+      <c r="C53" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>«Пересвет» — медцентр (4 филиала, КТ/МРТ)</t>
@@ -4173,7 +4185,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
@@ -4184,7 +4196,7 @@
       <c r="R53" t="inlineStr"/>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Резерв (верх ICP): 4 филиала + стационар, 47 врачей, 342 отзыва ПроДокторов, КТ/МРТ/пластика || Соцсети: ВК/TG заявлены на сайте, URL не подтверждены</t>
+          <t>Резерв (верх ICP): 4 филиала + стационар, 47 врачей, 342 отзыва ПроДокторов, КТ/МРТ/пластика || Соцсети: ВК/TG заявлены на сайте, URL не подтверждены || ОТПРАВЛЕНО 08.07 (сверка 09.07)</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4315,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Идея по записям для «Лоранж»</t>
+          <t>150–265 заявок в месяц салону: медиаплан для «Лоранж»</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4373,7 +4385,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Записи для двух филиалов «Океании»</t>
+          <t>Медиаплан для двух филиалов «Океании»</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4405,7 +4417,9 @@
       <c r="B57" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="C57" s="2" t="n"/>
+      <c r="C57" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>Институт красоты «Рашель»</t>
@@ -4453,7 +4467,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N57" s="2" t="n"/>
@@ -4464,7 +4478,7 @@
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="inlineStr">
         <is>
-          <t>С 2004, особняк купца Ерыкалова XIX в. в центре (Кирова 12) — бренд-фактура; полный цикл; отзывы смешанные (Zoon/2ГИС) — угол «репутация+трафик»; соцсети не найдены по сниппетам (не подтверждено)</t>
+          <t>С 2004, особняк купца Ерыкалова XIX в. в центре (Кирова 12) — бренд-фактура; полный цикл; отзывы смешанные (Zoon/2ГИС) — угол «репутация+трафик»; соцсети не найдены по сниппетам (не подтверждено) || ОТПРАВЛЕНО 08.07 (сверка 09.07)</t>
         </is>
       </c>
     </row>
@@ -4475,7 +4489,9 @@
       <c r="B58" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="C58" s="2" t="n"/>
+      <c r="C58" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
           <t>Языковая школа Дмитрия Никитина</t>
@@ -4523,7 +4539,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N58" s="2" t="n"/>
@@ -4534,7 +4550,7 @@
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr">
         <is>
-          <t>Яндекс «Хорошее место—2026», 4.9; 2ГИС 5.0; 3 локации; кембриджские экзамены; проекты для преподавателей; ЕСТЬ маркетинг-ящик; ВК vk.com/dnschoolclub; осн. email nikitindss@mail.ru</t>
+          <t>Яндекс «Хорошее место—2026», 4.9; 2ГИС 5.0; 3 локации; кембриджские экзамены; проекты для преподавателей; ЕСТЬ маркетинг-ящик; ВК vk.com/dnschoolclub; осн. email nikitindss@mail.ru || ОТПРАВЛЕНО 08.07 (сверка 09.07)</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4599,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Набор к сентябрю для LEO school</t>
+          <t>Заявки ×2,5 к сентябрю: медиаплан для LEO school</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -4653,7 +4669,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Свои пациенты для «Эталона»</t>
+          <t>14,6 ₽ выручки на 1 ₽ рекламы: медиаплан для «Эталона»</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -5566,7 +5582,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -5576,7 +5592,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -5586,7 +5602,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -5606,7 +5622,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9">
@@ -5626,7 +5642,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>0.07407407407407407</v>
+        <v>0.05714285714285714</v>
       </c>
     </row>
     <row r="11">
@@ -5740,7 +5756,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -5765,7 +5781,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -5790,7 +5806,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
@@ -5799,7 +5815,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.2</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -5859,7 +5875,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -5868,7 +5884,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0.125</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -5884,7 +5900,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -5893,7 +5909,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -5953,7 +5969,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -5962,7 +5978,7 @@
         <v>2</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>0.08</v>
+        <v>0.06060606060606061</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -6047,7 +6063,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C37" t="n">
         <v>0</v>
@@ -6056,7 +6072,7 @@
         <v>1</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -6072,7 +6088,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
@@ -6081,7 +6097,7 @@
         <v>1</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>0.0625</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -6194,13 +6210,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -6215,7 +6231,7 @@
         <v>2</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>0.0741</v>
+        <v>0.0571</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -6291,7 +6307,7 @@
         <v>71</v>
       </c>
       <c r="C2" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Run 11.07: no replies/bounces; reconcile 09.07 sends (Lorange double-send, Okeania with PDF decks, Uclinic, LEO; followups Klassik-Dent/Lika/Profieng; Star Talk nudge sent); 18 followup-1 drafts for 07-09.07 cohorts (fixed-price angle for medicine, Krasnodar x9 post for dental); batch-7 of 8 cold letters incl. FIX variant (EXP-004-fixprice); diff-review observations
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -1135,7 +1135,7 @@
       </c>
       <c r="N9" s="2" t="n"/>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="2" t="n"/>
       <c r="R9" t="inlineStr"/>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="N10" s="2" t="n"/>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="2" t="n"/>
       <c r="R10" t="inlineStr"/>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="N19" s="2" t="n"/>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="2" t="n"/>
       <c r="R19" t="inlineStr"/>
@@ -3995,7 +3995,9 @@
       <c r="B51" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="C51" s="2" t="n"/>
+      <c r="C51" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
           <t>Uclinic — клиника экспертной косметологии</t>
@@ -4043,7 +4045,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N51" s="2" t="n"/>
@@ -4054,7 +4056,7 @@
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr">
         <is>
-          <t>Резерв: премии ПроДокторов 2020/2021/2023, 498 отзывов, 14 врачей; своё приложение записи; InMode; направление «Косметология до 25 / Glow Club»; сильный собственный маркетинг — калибровать оффер || IG @uclinic.ru</t>
+          <t>Резерв: премии ПроДокторов 2020/2021/2023, 498 отзывов, 14 врачей; своё приложение записи; InMode; направление «Косметология до 25 / Glow Club»; сильный собственный маркетинг — калибровать оффер || IG @uclinic.ru || ОТПРАВЛЕНО 09.07; отправлена версия Яны на базе v4 (новый тред)</t>
         </is>
       </c>
     </row>
@@ -4245,17 +4247,17 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Рост с 33 до 191 заявки в месяц: медиаплан для Essenti</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mediaplan</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N54" s="2" t="n"/>
@@ -4266,7 +4268,7 @@
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Резерв на будущее (не дублировать Волгоград с Uclinic в одном батче)</t>
+          <t>Резерв на будущее (не дублировать Волгоград с Uclinic в одном батче) || БАТЧ №7: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4279,9 @@
       <c r="B55" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="C55" s="2" t="n"/>
+      <c r="C55" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
           <t>«Лоранж» — студия красоты</t>
@@ -4325,7 +4329,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N55" s="2" t="n"/>
@@ -4336,7 +4340,7 @@
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="inlineStr">
         <is>
-          <t>С 2003; 2ГИС 4.8 (285); «Лучший салон красоты 2023»; ~17 сотрудников; СПА/фитобочка/татуаж/инъекции; IG @lorange2003 1,7K; ВК заявлен, URL не подтверждён</t>
+          <t>С 2003; 2ГИС 4.8 (285); «Лучший салон красоты 2023»; ~17 сотрудников; СПА/фитобочка/татуаж/инъекции; IG @lorange2003 1,7K; ВК заявлен, URL не подтверждён || ОТПРАВЛЕНО 09.07; ДВОЙНАЯ ОТПРАВКА</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4351,9 @@
       <c r="B56" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="C56" s="2" t="n"/>
+      <c r="C56" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="D56" t="inlineStr">
         <is>
           <t>«Океания» Clinic &amp; SPA</t>
@@ -4395,7 +4401,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N56" s="2" t="n"/>
@@ -4406,7 +4412,7 @@
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr">
         <is>
-          <t>2 филиала (косметология Рабочая 29/39, SPA Валовая 2/10); ПроДокторов 14 врачей 209 отзывов; без выходных 9–21; несколько сайтов — распылённый digital; ВК/TG заявлены, URL не подтверждены</t>
+          <t>2 филиала (косметология Рабочая 29/39, SPA Валовая 2/10); ПроДокторов 14 врачей 209 отзывов; без выходных 9–21; несколько сайтов — распылённый digital; ВК/TG заявлены, URL не подтверждены || ОТПРАВЛЕНО 09.07; Яна отправила свою правку v4 новым письмом + приложила оба PDF-кейса</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4567,9 @@
       <c r="B59" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="C59" s="2" t="n"/>
+      <c r="C59" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>LEO school — центр допобразования</t>
@@ -4609,7 +4617,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Подготовлено</t>
+          <t>Отправлено</t>
         </is>
       </c>
       <c r="N59" s="2" t="n"/>
@@ -4620,7 +4628,7 @@
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr">
         <is>
-          <t>2 адреса + онлайн; 9 языков; летний интенсив ЕГЭ + лагерь; партнёр Liden&amp;Denz; РКИ, профориентация; ВК/TG не найдены по сниппетам (не подтверждено)</t>
+          <t>2 адреса + онлайн; 9 языков; летний интенсив ЕГЭ + лагерь; партнёр Liden&amp;Denz; РКИ, профориентация; ВК/TG не найдены по сниппетам (не подтверждено) || ОТПРАВЛЕНО 09.07; отправлен СТАРЫЙ черновик v2 (без медиаплан-CTA) — фикс-угол добавлен в фоллоу-ап</t>
         </is>
       </c>
     </row>
@@ -4739,17 +4747,17 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Заявок ×9 для одиночной стоматологии — расчёт для «Имплант Люкс»</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N61" s="2" t="n"/>
@@ -4760,7 +4768,7 @@
       <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr">
         <is>
-          <t>Резерв: ПроДокторов 11 врачей 137 отзывов, премии 2023/2024/2025; 2ГИС 4.9 (84); локомотив имплантация; с 2004; экс-главврач ушёл в 2025 — повод «перестройка маркетинга»</t>
+          <t>Резерв: ПроДокторов 11 врачей 137 отзывов, премии 2023/2024/2025; 2ГИС 4.9 (84); локомотив имплантация; с 2004; экс-главврач ушёл в 2025 — повод «перестройка маркетинга» || БАТЧ №7: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -4809,17 +4817,17 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Записи для City Clinic: бесплатный медиаплан</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mediaplan</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N62" s="2" t="n"/>
@@ -4830,7 +4838,7 @@
       <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr">
         <is>
-          <t>Резерв: 2ГИС 4.5 (94); с 2016; лазер+инъекции+аппаратная; ЛПР не найден (минус для холодного захода); IG @cityclinic38; ВК/TG заявлены в 2ГИС</t>
+          <t>Резерв: 2ГИС 4.5 (94); с 2016; лазер+инъекции+аппаратная; ЛПР не найден (минус для холодного захода); IG @cityclinic38; ВК/TG заявлены в 2ГИС || БАТЧ №7: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -4879,17 +4887,17 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ученики в 1–10 классы «Колибри» — набор 2026/27</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N63" s="2" t="n"/>
@@ -4900,7 +4908,7 @@
       <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr">
         <is>
-          <t>Резерв: набор в 1–10 классы на 2026–27 (один источник — сверить); 3 здания + детсад (экосистема сад→школа); полный день 8–19, английский с носителями; соцсети не найдены по сниппетам</t>
+          <t>Резерв: набор в 1–10 классы на 2026–27 (один источник — сверить); 3 здания + детсад (экосистема сад→школа); полный день 8–19, английский с носителями; соцсети не найдены по сниппетам || БАТЧ №7: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -5299,17 +5307,17 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Новые клиенты для LUNAMEL — 18 000 ₽</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>price18</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N69" s="2" t="n"/>
@@ -5320,7 +5328,7 @@
       <c r="R69" t="inlineStr"/>
       <c r="S69" t="inlineStr">
         <is>
-          <t>Резерв micro: Советская 54Б, 10 лет; маникюр/педикюр/брови/ресницы; ВК не подтверждён || Рекламная услуга для оффера: маникюр с покрытием</t>
+          <t>Резерв micro: Советская 54Б, 10 лет; маникюр/педикюр/брови/ресницы; ВК не подтверждён || Рекламная услуга для оффера: маникюр с покрытием || БАТЧ №7: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -5369,17 +5377,17 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Новые ученики для «Вокальной Мастерской» — 18 000 ₽</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>price18</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N70" s="2" t="n"/>
@@ -5390,7 +5398,7 @@
       <c r="R70" t="inlineStr"/>
       <c r="S70" t="inlineStr">
         <is>
-          <t>Резерв micro: центр города; вокал/гитара/фортепиано; хвалят преподавателя Ирину; ВК не подтверждён || Рекламная услуга для оффера: уроки вокала для взрослых (бесплатное пробное)</t>
+          <t>Резерв micro: центр города; вокал/гитара/фортепиано; хвалят преподавателя Ирину; ВК не подтверждён || Рекламная услуга для оффера: уроки вокала для взрослых (бесплатное пробное) || БАТЧ №7: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -5439,17 +5447,17 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ученики для «Лизетты» к осеннему набору</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mediaplan</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N71" s="2" t="n"/>
@@ -5460,7 +5468,7 @@
       <c r="R71" t="inlineStr"/>
       <c r="S71" t="inlineStr">
         <is>
-          <t>Резерв micro (на грани сегмента — 5 филиалов): первое занятие бесплатно || Рекламная услуга для оффера: курс рисования с нуля (первое бесплатно)</t>
+          <t>Резерв micro (на грани сегмента — 5 филиалов): первое занятие бесплатно || Рекламная услуга для оффера: курс рисования с нуля (первое бесплатно) || БАТЧ №7: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -5509,17 +5517,17 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ученики для 5 филиалов «Интер-Лэнг» — к сентябрю</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Резерв</t>
+          <t>Подготовлено</t>
         </is>
       </c>
       <c r="N72" s="2" t="n"/>
@@ -5530,7 +5538,7 @@
       <c r="R72" t="inlineStr"/>
       <c r="S72" t="inlineStr">
         <is>
-          <t>Резерв (сильный, 5/5): 5+ филиалов по районам (2ГИС подтверждает) — идеально под геотаргет; 3000+ учеников/год; линейка: английский/китайский/ментальная арифметика/скорочтение — сегментация кампаний; ВК/TG заявлены, URL не подтверждены</t>
+          <t>Резерв (сильный, 5/5): 5+ филиалов по районам (2ГИС подтверждает) — идеально под геотаргет; 3000+ учеников/год; линейка: английский/китайский/ментальная арифметика/скорочтение — сегментация кампаний; ВК/TG заявлены, URL не подтверждены || БАТЧ №7: отправка вт 14.07</t>
         </is>
       </c>
     </row>
@@ -5582,7 +5590,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -5592,7 +5600,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -5602,7 +5610,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
@@ -5622,7 +5630,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9">
@@ -5642,7 +5650,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>0.05714285714285714</v>
+        <v>0.05128205128205128</v>
       </c>
     </row>
     <row r="11">
@@ -5756,7 +5764,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -5806,7 +5814,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
@@ -5815,7 +5823,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.2</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -5875,7 +5883,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -5884,7 +5892,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -5900,7 +5908,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -5909,7 +5917,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.04545454545454546</v>
+        <v>0.04</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -5969,7 +5977,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -5978,7 +5986,7 @@
         <v>2</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>0.06060606060606061</v>
+        <v>0.05405405405405406</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -6088,7 +6096,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
@@ -6097,7 +6105,7 @@
         <v>1</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>0.04545454545454546</v>
+        <v>0.03846153846153846</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -6210,13 +6218,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -6231,7 +6239,7 @@
         <v>2</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>0.0571</v>
+        <v>0.0513</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -6307,7 +6315,7 @@
         <v>71</v>
       </c>
       <c r="C2" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
@@ -6350,7 +6358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6450,27 +6458,64 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>EXP-004-fixprice</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Оффер «заявки по фиксированной цене из альтернативного источника» (пост Яны: одиночные клиники vs сети, SMS-валидация, кейс Краснодар ×9) даст больше ответов в медицине/образовании, чем универсальное письмо про рекламу</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>основной оффер письма</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FIX — фикс-цена как главный оффер (Имплант Люкс, Интер-Лэнг, Колибри + фикс-крупица в мед-фоллоу-апах)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>mediaplan — медиаплан-CTA v4 (остальные)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>REDESIGN-v2</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Полная переработка системы по итогам аудита (59 находок): подтверждение отправки, статусы v2, Asana-интеграция, A/B, когортная аналитика, надёжность запусков</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>sales-agent/*</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
         <is>
           <t>применено</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>исчезнут потерянные лиды и невидимые ответы; появится измеримый цикл улучшения стратегии</t>
         </is>

</xml_diff>

<commit_message>
Batch 8 (FIX focus per Yana): 10 new leads from 3 research agents (4 medicine/dental, 3 education, 3 laser hair removal), fixed-price-lead letters in outbox (Gmail connector needs reauth, drafts deferred); multichannel D+2 DM cadence
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S72"/>
+  <dimension ref="A1:S82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5539,6 +5539,706 @@
       <c r="S72" t="inlineStr">
         <is>
           <t>Резерв (сильный, 5/5): 5+ филиалов по районам (2ГИС подтверждает) — идеально под геотаргет; 3000+ учеников/год; линейка: английский/китайский/ментальная арифметика/скорочтение — сегментация кампаний; ВК/TG заявлены, URL не подтверждены || БАТЧ №7: отправка вт 14.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C73" s="2" t="n"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Центр стоматологии и имплантологии «Астра-мед»</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Пермь</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Кузнецова Ирина Михайловна (гендиректор и единственный учредитель)</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>astramed-priem@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://астрамедцентр.рф/</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Заявок ×9 для одиночной стоматологии — расчёт для «Астра-мед»</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="n"/>
+      <c r="P73" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q73" s="2" t="n"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Цифровая имплантология; 6 врачей/47 отзывов ПроДокторов, 4.8/150 2ГИС; живут на агрегаторах; на сайте опубликован личный email директора kuznecovane@mail.ru (запасной контакт); стоматолог-микроскопист Ольга Перцовская (25 лет стажа) || confidence 5/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C74" s="2" t="n"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника «Д'Арт»</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Воронеж</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Левченко Давид Михайлович (учредитель и главврач); директор Миликова Елена Алексеевна</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>dave3d@rambler.ru</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://клиника-дарт.рф/</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Заявок ×9 для одиночной стоматологии — расчёт для «Д'Арт»</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="n"/>
+      <c r="P74" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q74" s="2" t="n"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Имплантация/протезирование/виниры в тайтле; 36 отзывов ПроДокторов; врач Провоторов А.В. 13 персональных отзывов — идут «на врача»; email на rambler — устаревший digital; юрлицо с 2003 || confidence 4/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C75" s="2" t="n"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Стоматология «ИАТРОС»</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Волгоград</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Худавердян Дереник Бениаминович (директор, вероятно врач-собственник)</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>iatros34@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://iatros34.ru/</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Заявок ×9 для одиночной стоматологии — расчёт для «ИАТРОС»</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="n"/>
+      <c r="P75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" s="2" t="n"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Победитель премии ПроДокторов 2020 и 2024; 10 врачей/69 отзывов; имплантация+ортодонтия+детская; без выходных 9–20:30 — есть мощности; зависимость от агрегатора || confidence 5/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C76" s="2" t="n"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Первая гинекологическая клиника</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Красноярск</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Логиновский Андрей Сергеевич (директор, сам врач клиники)</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>firstgc@mail.ru</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://firstgc.ru/</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Пациентки по фиксированной цене заявки — расчёт для «Первой гинекологической»</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="n"/>
+      <c r="P76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="2" t="n"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Гинекология/УЗИ/кольпоскопия; 4.8/348 2ГИС; правобережье (Белые росы, Карамзина 18); именные врачи с лояльной базой (Морозова, Дресвянская, Астафьева); живут на агрегаторах || confidence 4/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Лингвистический центр LEXXIS</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>admin@lexxis.ru</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://lexxis.ru/</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Ученики по фиксированной цене заявки — к сентябрю для LEXXIS</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="n"/>
+      <c r="P77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="2" t="n"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>2 филиала по районам (Ключевская 15 ВИЗ, Куйбышева 21 центр) + Первоуральск; 4.5/45 2ГИС; официальный центр Кембриджских экзаменов (KET–CPE) и Pearson — длинный LTV, учатся семьями; запасной email lexxis-ekb@lexxis.ru || confidence 4/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Частная школа «РОСТ»</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Воробьева Олеся Вячеславовна (директор АНО «ОЦ «Рост»)</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>info@rost21vek.ru</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://rost21vek.ru/</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Заявки в 1-е классы по фиксированной цене — для школы «РОСТ»</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="n"/>
+      <c r="P78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="2" t="n"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Школа полного дня 8–19, ~140 учеников, классы до 16; из-за наплыва открыли ТРЕТИЙ первый класс на 2025–26 — набор горячий; ЖК «Жуковка» (Победы 55/1); учредители Риттер М.В. и Бойко А.В.; чек за 11 лет обучения — максимальный LTV || confidence 5/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Детский центр развития «Яркие Дети» (Казань)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Казань</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>yarkiedeti.kzn@yarkiedeti.ru</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://kazan.yarkiedeti.ru/</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Заявки по фиксированной цене для трёх филиалов «Ярких Детей»</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="n"/>
+      <c r="P79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="2" t="n"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>3 филиала по районам Казани; 5.0/152 2ГИС; локомотивы: скорочтение, ментальная арифметика, продлёнка (пик к сентябрю); преподаватели по именам в отзывах (Павел, Татьяна); франчайзи-филиалы, не сам бренд || confidence 4/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Ларейн — центр лазерной косметологии</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Мартынова Наталья Анатольевна (директор ООО «Ларейн»; владелец Мартынова Людмила Васильевна)</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>lareine@bk.ru</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://lareine.ru/</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Заявки на эпиляцию по 504 ₽ с оплатой за результат — расчёт для «Ларейн»</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="n"/>
+      <c r="P80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="2" t="n"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Александрит + диод; «лучшая клиника лазерной эпиляции Екб» в отзывах; 4.7/31 Doctu + ~300 оценок xtool; с 2013, одна точка (Декабристов 75); директор сменилась 04.2025 — момент для захода; продвижение только карты; IG @lareine_clinic (не подтверждено) || confidence 5/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>МЦ «Лазер плюс Эстетика»</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Самара</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Вьюгина Светлана Владимировна (директор, соучредитель с Яруллиной Р.М.)</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>laser-2012@mail.ru</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://www.laser-estetik.ru/</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Заявки на эпиляцию по 504 ₽ с оплатой за результат — расчёт для «Лазер плюс Эстетика»</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="n"/>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" s="2" t="n"/>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>Александритовый лазер, эпиляция от 500 ₽ — готовый оффер; 2 точки (Кирова 316 + ТЦ Перекресток); 23 отзыва/9 врачей ПроДокторов, отзывы 2025; с 2012; новые — по сарафану и картам || confidence 5/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C82" s="2" t="n"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Клиника лазерной косметологии +</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Пермь</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Акбашева Светлана Шамсиевна (гендиректор, с 2018)</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>cliniclaser@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://cliniclaser.ru/</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Заявки на эпиляцию по 504 ₽ с оплатой за результат — расчёт для вашей клиники</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="n"/>
+      <c r="P82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q82" s="2" t="n"/>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>Диодный MeDioStar Effect (Asclepion); 4.9/148 2ГИС при 3.7/25 Фламп — разрыв под формат «трафик+репутация»; врачи-дерматокосметологи; программа лояльности 300 баллов; одна точка (Пушкина 80) || confidence 5/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
         </is>
       </c>
     </row>
@@ -5580,7 +6280,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4">
@@ -5590,7 +6290,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -6312,7 +7012,7 @@
         <v>46209</v>
       </c>
       <c r="B2" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C2" t="n">
         <v>39</v>

</xml_diff>

<commit_message>
Batch 9: 20 single-practice dental clinics across 20 cities (5 research agents), personalized HTML drafts in Gmail split across three designs (7 chat / 7 P&L dashboard / 6 schedule journal), EXP-005-design launched, phones captured for TG follow-ups
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S82"/>
+  <dimension ref="A1:S102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6239,6 +6239,1406 @@
       <c r="S82" t="inlineStr">
         <is>
           <t>Диодный MeDioStar Effect (Asclepion); 4.9/148 2ГИС при 3.7/25 Фламп — разрыв под формат «трафик+репутация»; врачи-дерматокосметологи; программа лояльности 300 баллов; одна точка (Пушкина 80) || confidence 5/5 || БАТЧ №8 (FIX, чт 16.07): текст письма в outbox/2026-07-11-batch8-fix.md; Gmail-черновик создать после реавторизации коннектора</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Клиника эстетической стоматологии «Галадент» (ООО «КЭС «Галадент»)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Уфа</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Сарваров Ильдус Марианович, генеральный директор и единственный учредитель (с 2005 г., rusprofile.ru)</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>galadent-ufa@mail.ru</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://galadent.ru/</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Короткий диалог о пациентах для «Галадент»</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>V2-chat</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="n"/>
+      <c r="P83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q83" s="2" t="n"/>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>21 врач и 610 отзывов на ПроДокторов — врачи клиники стали лауреатами премии ПроДокторов 2024 • Работает с ноября 2005 года, штат вырос до 34-35 сотрудников (rusprofile) • Маржинальные направления-локомотивы: ортодонтия, протезирование, хирургия и челюстно-лицевая хирургия • График до 21:00 (пн-пт с 9:00, сб с 11:00) — активно представлена на ПроДокторов, 2ГИС, НаПоправку, doctu.ru || confidence 5/5 || БАТЧ №9 (HTML-дизайн V2-chat): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Центр Дентальной Имплантации</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Томск</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Ворочилов Виталий Викторович — генеральный директор и единственный учредитель ООО «ЦДИ» (rusprofile.ru, ИНН 7017266114)</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>cdistom@mail.ru</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://cdistom.ru/</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Короткий диалог о пациентах для Центра Дентальной Имплантации</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>V2-chat</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="n"/>
+      <c r="P84" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q84" s="2" t="n"/>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>Одиночная клиника на ул. Говорова, 19В ст.1, работает с 2010 года (15 лет на рынке), директор бессменно с 2014 года • 9 врачей и 130 отзывов на ПроДокторов, рейтинг 4.6 на 2ГИС — карточки активно ведутся на ПроДокторов, 2ГИС, Фламп, doctu.ru (зависимость от агрегаторов) • Локомотив — имплантация и протезирование: пациенты в отзывах хвалят хирургов-имплантологов Штина Валентина Игоревича и Синдяка  || confidence 5/5 || БАТЧ №9 (HTML-дизайн V2-chat): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника «София»</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Таганрог</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Кудрявцев Михаил Игоревич, генеральный директор ООО «София» (ИНН 6154149636, сниппет rusprofile.ru/spark-interfax.ru)</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>sofdent@bk.ru</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://sofia-taganrog.ru/</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Короткий диалог о пациентах для «Софии»</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>V2-chat</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="n"/>
+      <c r="P85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" s="2" t="n"/>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>6 врачей и 94 отзыва на ПроДокторов — живая одиночная клиника нужного размера, единственный адрес: ул. Ленина, 205 • Маржинальные услуги: протезирование, имплантация, эстетика — при этом консультация от 500 руб. (по данным 32top) — есть потенциал роста среднего чека • Зависимость от агрегаторов: активные карточки на ПроДокторов, 2ГИС, 32top, Яндекс.Картах — основной канал репутации, а не собственн || confidence 5/5 || БАТЧ №9 (HTML-дизайн V2-chat): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Стоматология «Меди Лайт» (ООО «Меди Лайт»)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Рязань</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Ковальчук Елена Александровна, директор ООО «Меди Лайт» (rusprofile.ru, ИНН 6234108434)</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>medilicht@mail.ru</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://medi-light.ru/</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Короткий диалог о пациентах для «Меди Лайт»</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>V2-chat</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="n"/>
+      <c r="P86" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="2" t="n"/>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Независимая клиника, работает с октября 2012 года (13+ лет), ООО «Меди Лайт», уставный капитал 10 000 руб. • На ПроДокторов: площадка на 2-й Линии — 16 врачей и 275 отзывов; профили также на СберЗдоровье (DocDoc) и Яндекс.Картах — заметная зависимость от агрегаторов • Филиал на Татарской, 20 помечен на ПроДокторов как «на ремонте» — хороший повод для разговора о загрузке основной площадки • Маржин || confidence 4/5 || БАТЧ №9 (HTML-дизайн V2-chat): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C87" s="2" t="n"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Стоматологический центр «Лина»</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Мытищи</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Егоров Евгений Владиславович, генеральный директор ООО «Лина» (ИНН 5029182264, rusprofile.ru)</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>dantist@linadent.ru</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://linadent.ru/</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Короткий диалог о пациентах для центра «Лина»</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>V2-chat</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="n"/>
+      <c r="P87" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q87" s="2" t="n"/>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>16 врачей и 49 отзывов на ПроДокторов — типичная одиночная клиника среднего размера, живой поток пациентов • Работает по ОМС Московской области с 01.02.2017 — микс бюджетного и коммерческого потока, есть куда растить платные направления • Маржинальные услуги: имплантация «под ключ» (диагностика + работа врача + коронка) и протезирование • Сильная зависимость от агрегаторов: карточки на 2ГИС, Zoon, || confidence 5/5 || БАТЧ №9 (HTML-дизайн V2-chat): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника «Азурит»</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Астрахань</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>azuritsk@mail.ru</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://azurit30.ru/</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Короткий диалог о пациентах для «Азурита»</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>V2-chat</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="n"/>
+      <c r="P88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="2" t="n"/>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Штат 10 врачей по ПроДокторов (в карточке 2ГИС заявлено 16 сертифицированных врачей) — верх целевого диапазона, один адрес: ул. Красная Набережная, 39/1 • Полный набор маржинальных направлений: имплантация, взрослая и детская ортодонтия, протезирование, лазерная стоматология • Рейтинг 4.5 на 2ГИС при 141 отзыве, но лишь 12 отзывов на ПроДокторов — репутация размазана по агрегаторам (2ГИС, Zoon, 32 || confidence 4/5 || БАТЧ №9 (HTML-дизайн V2-chat): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C89" s="2" t="n"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Стоматология «НоваДэнт»</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Тула</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>info.novadent71@gmail.com</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://www.dent-tula.ru/</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Короткий диалог о пациентах для «НоваДэнт»</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>V2-chat</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="n"/>
+      <c r="P89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q89" s="2" t="n"/>
+      <c r="R89" t="inlineStr"/>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Одиночная Hi-tech 3D-клиника в центре Тулы (ул. Демонстрации, д. 1-Г, ТЦ «УтюгЪ», 4 этаж), 8 врачей — на ПроДокторов 74 отзыва • Победитель премии ПроДокторов 2024, 2023, 2022 и 2020 годов — сильная зависимость репутации от агрегатора • Присутствует сразу на нескольких агрегаторах: ПроДокторов, Startsmile, Dentalworld, 32top • Маржинальные услуги: имплантация за одно посещение, цены на ПроДокторов || confidence 4/5 || БАТЧ №9 (HTML-дизайн V2-chat): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C90" s="2" t="n"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Sahar.Dental — центр дентальной имплантации и стоматологии</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Челябинск</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>plan@sahar.dental</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://sahar.dental/</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Sahar.Dental: сколько стоит пациент и сколько он приносит</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>V3-pnl</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="n"/>
+      <c r="P90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="2" t="n"/>
+      <c r="R90" t="inlineStr"/>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Профильный центр дентальной имплантации: более 20 000 операций по имплантации, более 20 лет практики • 12 врачей и 129 отзывов на ПроДокторов, плюс 208 отзывов на 2ГИС — сильная зависимость от агрегаторов • Одна локация: Челябинск, ул. Советская, 38 (Центральный район) • График: пн-пт 09:00-21:00, сб-вс 09:00-19:00 — работает без выходных || confidence 4/5 || БАТЧ №9 (HTML-дизайн V3-pnl): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C91" s="2" t="n"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Центр стоматологии «Сапфир»</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Красноярск</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Поляков Роман Анатольевич — генеральный директор ООО «ЦС Сапфир» (rusprofile.ru, ИНН 2465162135) и практикующий стоматолог-ортопед клиники</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>sapfir.stom@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://sapfircs.ru/</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>«Сапфир»: сколько стоит пациент и сколько он приносит</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>V3-pnl</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="n"/>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" s="2" t="n"/>
+      <c r="R91" t="inlineStr"/>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Рейтинг 4.9 при 146 отзывах на 2ГИС, 8 врачей на ПроДокторов, 54 отзыва (4.9) на doctu.ru — активные карточки на Zoon, Фламп, 2ГИС, ПроДокторов • Маржинальные направления: имплантация «под ключ» от одного зуба до полной челюсти по протоколам All-on-4/All-on-6 на премиальных системах Straumann, Dentium, Inno • Владелец = врач: директора Полякова Р.А. и имплантолога Шишлова П.А. пациенты поимённо хв || confidence 5/5 || БАТЧ №9 (HTML-дизайн V3-pnl): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Стоматология 32</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Омск</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Потапов Александр Геннадьевич — генеральный директор ООО «Стоматология 32» (rusprofile.ru, ИНН 5504071659)</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>info@stoma-32.ru</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://stoma-32.ru/</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>«Стоматология 32»: сколько стоит пациент и сколько он приносит</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>V3-pnl</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="n"/>
+      <c r="P92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" s="2" t="n"/>
+      <c r="R92" t="inlineStr"/>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>12 врачей высшей категории, рейтинг 4.9 на 32top; отзывы также на ПроДокторов (9), Zoon (20) и Фламп — сильная зависимость от агрегаторов • Тяжёлое оснащение под маржинальные направления: собственные компьютерные томографы, зуботехническая лаборатория, микроскопы Carl Zeiss, навигационная имплантация; в штате имплантолог, ортопед и ортодонт • Старожил рынка: ООО зарегистрировано в декабре 2002 год || confidence 4/5 || БАТЧ №9 (HTML-дизайн V3-pnl): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Дента Клиник (стоматология на Северном)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Ростов-на-Дону</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Дургалян Петрос Ервандович, директор</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>denta-clinic24@mail.ru</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://denta-clinic24.ru/</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>«Дента Клиник»: сколько стоит пациент и сколько он приносит</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>V3-pnl</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="n"/>
+      <c r="P93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q93" s="2" t="n"/>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Одиночная районная клиника в спальном районе Северный (пр-т Космонавтов, 46), работает без выходных: будни 09:00-20:00, сб-вс 10:00-15:00 • Маржинальные направления: имплантация, ортопедия (протезирование), пародонтология, детская стоматология • Рейтинг 4.8 на 2ГИС (20 оценок), при этом всего 20 оценок — репутационный объём заметно ниже конкурентов, есть точка роста • Сильная зависимость от агрега || confidence 4/5 || БАТЧ №9 (HTML-дизайн V3-pnl): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника «Союз»</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Брянск</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Грибанов Сергей Михайлович, директор ООО «Союз» (rusprofile.ru, ИНН 3250526923)</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>soyz32@ya.ru</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://soyz32.ru/</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>«Союз»: сколько стоит пациент и сколько он приносит</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>V3-pnl</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="n"/>
+      <c r="P94" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q94" s="2" t="n"/>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>Одиночная клиника на ул. Дуки, 47 к1: 24 врача и 209 отзывов на ПроДокторов — верхняя граница целевого размера, при этом одна локация • ООО «Союз» работает с октября 2011 года (14+ лет на рынке) • Маржинальные направления: имплантация, ортодонтия, лечение под микроскопом, лазерная стоматология, 3D-рентген-диагностика • Разрозненное присутствие на агрегаторах (ПроДокторов, 2ГИС, 32top, big-book-med || confidence 4/5 || БАТЧ №9 (HTML-дизайн V3-pnl): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C95" s="2" t="n"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника SmileDent (Смайл Дент)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Подольск</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Скалькович Артем Валерьевич, генеральный директор ООО «СМАЙЛ ДЕНТ» (ИНН 5036136290, spark-interfax/реестры)</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>info@smiledent32.ru</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://smiledent32.ru/</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>SmileDent: сколько стоит пациент и сколько он приносит</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>V3-pnl</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="n"/>
+      <c r="P95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" s="2" t="n"/>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>Одиночная клиника, работает с 2014 года (ООО зарегистрировано 24.12.2013, ул. Профсоюзная, 7А), 2 совладельца — классический собственнический бизнес • На ПроДокторов карточка «Смайл дент»: 17 врачей и 171 отзыв — живая клиника в целевом диапазоне 5–30 врачей • Маржинальные направления: имплантация «под ключ» с костной пластикой, протезирование (коронки, мосты), ортодонтия, виниры • Зависимость от  || confidence 4/5 || БАТЧ №9 (HTML-дизайн V3-pnl): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C96" s="2" t="n"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника Dentus (Дентус)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Пигулевский Дмитрий Александрович, генеральный директор ООО «Питерстом» (юрлицо клиники Dentus)</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>mail@dentusclinic.ru</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://dentusclinic.ru/</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Dentus: сколько стоит пациент и сколько он приносит</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>V3-pnl</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="n"/>
+      <c r="P96" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q96" s="2" t="n"/>
+      <c r="R96" t="inlineStr"/>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>Одиночная клиника в спальном ЖК «Юбилейный квартал» (Комендантский пр., 53 к1): 9 врачей и 295 отзывов на ПроДокторов • 835 отзывов и рейтинг 5.0 на 2ГИС, 4.5 на Zoon — сильная зависимость репутации и трафика от агрегаторов (2ГИС, Zoon, НаПоправку, InfoDoctor, 32top) • Полный набор маржинальных направлений: имплантация, протезирование всех типов, ортодонтия (брекеты), 4 кабинета включая хирургичес || confidence 5/5 || БАТЧ №9 (HTML-дизайн V3-pnl): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C97" s="2" t="n"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Центр стоматологии «Дельта» (юрлицо ООО «Смайл Плюс», ИНН 5610257172)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Оренбург</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>stomdelta56@ya.ru</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://delta-56.ru/</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Журнал записи «Дельты» без окон — расчёт</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>V5-schedule</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="n"/>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" s="2" t="n"/>
+      <c r="R97" t="inlineStr"/>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>6 врачей и 147 отзывов на ПроДокторов — основной канал репутации, плюс карточки в 2ГИС и Яндекс.Картах • Полный цикл: терапия, хирургия, имплантация и протезирование — маржинальные направления заявлены на сайте отдельными разделами • Работает ежедневно с 9:00 до 21:00 без выходных • Одна локация в центре города: ул. Максима Горького, 22а || confidence 4/5 || БАТЧ №9 (HTML-дизайн V5-schedule): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C98" s="2" t="n"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Центральная стоматология им. Е.А. Беззубова (ООО «Центральная стоматология»)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Тольятти</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Беззубова Елена Анатольевна, директор ООО «Центральная стоматология»</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>cs_tlt@mail.ru</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://xn----7sbabph0atdigcpcbvwlhd3ethzcm.xn--p1acf/</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Журнал записи «Центральной стоматологии» без окон — расчёт</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>V5-schedule</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="n"/>
+      <c r="P98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q98" s="2" t="n"/>
+      <c r="R98" t="inlineStr"/>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>Именная клиника, работает с 2011 года; директор Елена Беззубова — клиника названа в честь Е.А. Беззубова • 7-8 стоматологов (32top), 75 отзывов на ПроДокторов — присутствие также на Zoon и 2ГИС • Полный спектр от лечения кариеса до имплантации, консультация от 1500 руб. • График: пн-пт 9:00-20:00, сб 9:00-19:00; адрес — ул. Ленина, 106 || confidence 4/5 || БАТЧ №9 (HTML-дизайн V5-schedule): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C99" s="2" t="n"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Стоматологический центр «Аполлония»</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Барнаул</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Маслов Виктор Владимирович — директор ООО «Стоматологический центр «Аполлония» (rusprofile.ru, ИНН 2222801559)</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>apolloniia-reg@bk.ru</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://apollonia-dent.ru/</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Журнал записи «Аполлонии» без окон — расчёт</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>V5-schedule</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="n"/>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q99" s="2" t="n"/>
+      <c r="R99" t="inlineStr"/>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>10 врачей и 36 отзывов на ПроДокторов, одна локация на ул. Малахова, 154Б; компания работает с 2012 года • Полный цикл маржинальных услуг: имплантация, ортодонтия, протезирование + собственная зуботехническая лаборатория (взрослое и детское отделения) • В отзывах на 2ГИС поимённо хвалят ортодонта Ольгу Борисовну (выравнивание зубов) и терапевта Воронину Викторию Викторовну — карточки ведутся на 2Г || confidence 4/5 || БАТЧ №9 (HTML-дизайн V5-schedule): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C100" s="2" t="n"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника «Современник»</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Ставрополь</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>sovremennik.stv26@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://sovremennik26.com/</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Журнал записи «Современника» без окон — расчёт</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>V5-schedule</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="n"/>
+      <c r="P100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q100" s="2" t="n"/>
+      <c r="R100" t="inlineStr"/>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>Команда из 5 специалистов: главврач-терапевт Фролова О.В., хирург Писарев С.Ю., гнатолог-ортопед Эльканов А.А., ортодонт Максимов Н.Д., пародонтолог Кожемякина А.П. • Маржинальные направления: имплантация, синус-лифтинг, микропротезирование, ортодонтия, гнатология — редкая для Ставрополя специализация • Всего 4 отзыва на ПроДокторов при 8877 отзывах у конкурентов города — клиника почти невидима на || confidence 3/5 || БАТЧ №9 (HTML-дизайн V5-schedule): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C101" s="2" t="n"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Клиника современной стоматологии «RedWhite»</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Тверь</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>info@klinika-redwhite.com</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://klinika-redwhite.com/</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Журнал записи RedWhite без окон — расчёт</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>V5-schedule</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="n"/>
+      <c r="P101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q101" s="2" t="n"/>
+      <c r="R101" t="inlineStr"/>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>Одиночная клиника на Волоколамском пр., 25 к1: 6 врачей, 57 отзывов на ПроДокторов, приём ежедневно 9:00–20:00 • Живые отзывы 2025 года: свежий кейс по имплантации Dentium на ПроДокторов (клиника вернула пациенту 34 000 руб. при осложнении) — репутация в агрегаторах критична • Имплантация на премиальных системах Astra Tech (Швеция) и MIS (Израиль), работа «в 4 руки» по американским протоколам — ма || confidence 3/5 || БАТЧ №9 (HTML-дизайн V5-schedule): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C102" s="2" t="n"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Клиника «Невская Стоматология»</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>info@nevstoma.ru</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://nevstoma.ru/</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Журнал записи «Невской Стоматологии» без окон — расчёт</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>V5-schedule</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="n"/>
+      <c r="P102" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q102" s="2" t="n"/>
+      <c r="R102" t="inlineStr"/>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>Одиночная клиника в спальном Невском районе, 6 врачей (ПроДокторов), включая челюстно-лицевого хирурга и стоматолога-имплантолога • Маржинальные направления: имплантация на системах Imlay и MIS C1, протезирование, эстетическая реставрация • Рейтинг 4.5 на НаПоправку (30 отзывов), но всего 5 отзывов на ПроДокторов — очевидный разрыв в управлении репутацией, точка входа для агентства • Публичный моб || confidence 4/5 || БАТЧ №9 (HTML-дизайн V5-schedule): отправка вт 15.07 / ср 16.07</t>
         </is>
       </c>
     </row>
@@ -6280,7 +7680,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -6290,7 +7690,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>34</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -6964,7 +8364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7034,7 +8434,7 @@
         <v>46216</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -7046,6 +8446,24 @@
         <v>0</v>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7058,7 +8476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7221,6 +8639,43 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EXP-005-design</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>HTML-письма с интерфейсными метафорами (чат/P&amp;L-дашборд/журнал записи) дают больше ответов от стоматологий, чем plain-text</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>дизайн письма</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>V2-chat (7)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>V3-pnl (7)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Batch 10: 10 multichannel leads (email + VK/TG/mobile pairs) with FIX drafts in Gmail; VK enrichment for batch-9 (2 verbatim links, env-limited); multichannel outreach table (51 leads, ready-to-send VK/TG texts) delivered
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCebmL2vZr5fxvaGcjjXKH
</commit_message>
<xml_diff>
--- a/sales-agent/report/report.xlsx
+++ b/sales-agent/report/report.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S102"/>
+  <dimension ref="A1:S112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7639,6 +7639,706 @@
       <c r="S102" t="inlineStr">
         <is>
           <t>Одиночная клиника в спальном Невском районе, 6 врачей (ПроДокторов), включая челюстно-лицевого хирурга и стоматолога-имплантолога • Маржинальные направления: имплантация на системах Imlay и MIS C1, протезирование, эстетическая реставрация • Рейтинг 4.5 на НаПоправку (30 отзывов), но всего 5 отзывов на ПроДокторов — очевидный разрыв в управлении репутацией, точка входа для агентства • Публичный моб || confidence 4/5 || БАТЧ №9 (HTML-дизайн V5-schedule): отправка вт 15.07 / ср 16.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C103" s="2" t="n"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Стоматология «Зангари»</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Ижевск</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>zangaristom@yandex.ru</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://zangaristom.ru</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Заявок ×9 для одиночной стоматологии — расчёт для «Зангари»</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="n"/>
+      <c r="P103" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q103" s="2" t="n"/>
+      <c r="R103" t="inlineStr"/>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>Семейная клиника 20+ лет, один адрес (Четырнадцатая 56а); ведут SEO-блог (статьи 2025); 19 отзывов 2ГИС; протезирование/элайнеры/имплантация || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C104" s="2" t="n"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника «Астра»</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Владимир</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Скоропад Эдуард Витальевич (хирург-имплантолог, владелец; практикует с 1983)</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>skoropad.eduard@rambler.ru</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://astra33.ru</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Заявок ×9 для одиночной стоматологии — расчёт для «Астры»</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="n"/>
+      <c r="P104" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" s="2" t="n"/>
+      <c r="R104" t="inlineStr"/>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>ЛИЧНАЯ почта врача-владельца — письмо минует администратора; хирургия/имплантация; мобильный публичный || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C105" s="2" t="n"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Клиника доктора Евграфова «Стоматолог»</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Медицина</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Курск</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Евграфов (врач-основатель, именная клиника)</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>stomatolog.12@mail.ru</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://stomatolog-kursk.ru</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Заявок ×9 для одиночной стоматологии — расчёт для клиники доктора Евграфова</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N105" s="2" t="n"/>
+      <c r="P105" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q105" s="2" t="n"/>
+      <c r="R105" t="inlineStr"/>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>10 врачей, 78 отзывов ПроДокторов; без выходных 9-20; мобильный публичный || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C106" s="2" t="n"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Студия лазерной эпиляции «Олива»</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Чебоксары</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>laser_oliva@mail.ru</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>http://laser-oliva.tilda.ws</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Заявки на эпиляцию по 504 ₽ с оплатой за результат — для «Оливы»</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="n"/>
+      <c r="P106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q106" s="2" t="n"/>
+      <c r="R106" t="inlineStr"/>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>3 точки; сайт — бесплатный Tilda-лендинг (точка роста); абонементы −10/−15/−20% (LTV-механика есть); мобильный владельца || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C107" s="2" t="n"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Клиника лазерной медицины «Возрождение»</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Киров</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>lazer-kirov@mail.ru</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://www.lazer-kirov.ru</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Заявки на эпиляцию по 504 ₽ с оплатой за результат — для «Возрождения»</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="n"/>
+      <c r="P107" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" s="2" t="n"/>
+      <c r="R107" t="inlineStr"/>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>Мед-клиника: 24 врача/41 отзыв ПроДокторов, лицензии; в ВК дают скидку 10% подписчикам — ценят соцсети, нет системного трафика; александрит || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C108" s="2" t="n"/>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Студия лазерной эпиляции «Волос нет»</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Бьюти</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Липецк</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>volosnet.lip@ya.ru</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://volos-net.clients.site</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Заявки на эпиляцию по 504 ₽ с оплатой за результат — для «Волос нет»</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="n"/>
+      <c r="P108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" s="2" t="n"/>
+      <c r="R108" t="inlineStr"/>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>Сайта нет (clients.site), запись через Dikidi; ВК и TG упомянуты в 2ГИС без URL; мобильный основной; без выходных || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C109" s="2" t="n"/>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Speak! English</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Хабаровск</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Стукалова Анастасия Владимировна (учредитель)</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>speakenglish27@mail.ru</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://speakenglish27.ru</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Ученики к сентябрю для Speak! English — бесплатный медиаплан</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="n"/>
+      <c r="P109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" s="2" t="n"/>
+      <c r="R109" t="inlineStr"/>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>С 2012, лицензия, международные экзамены; БЦ Феликс-Сити; мобильный публичный || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C110" s="2" t="n"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>ЧОУ «Новая школа Натальи Колгановой»</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Липецк</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Колганова Наталья Евгеньевна (директор)</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>info@kolganovaschool.ru</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://kolganovaschool.ru</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Ученики в «Новую школу» к сентябрю — бесплатный медиаплан</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="n"/>
+      <c r="P110" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" s="2" t="n"/>
+      <c r="R110" t="inlineStr"/>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Школа полного дня; набор на вечернюю подготовку 5-6 лет (отдельные посадочные); ЧОУ с 2021, лицензия; мобильный || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C111" s="2" t="n"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>АНОО «Академия Ростум»</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Пенза</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Завитаева Инна Викторовна (директор); основатель ГК — Александр Мухин</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>academy@rostum.ru</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://rostum.ru</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Ученики для 5 филиалов «Академии Ростум» — бесплатный медиаплан</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N111" s="2" t="n"/>
+      <c r="P111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" s="2" t="n"/>
+      <c r="R111" t="inlineStr"/>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>Первая частная школа области с лицензией; 5 адресов по Пензе; основатель медийный (АиФ, penzavzglyad) || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C112" s="2" t="n"/>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Центр развития ребенка «АБВГДейка»</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Пермь</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>info@abvgd-ka.ru</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://abvgd-ka.ru</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Ученики к сентябрю для «АБВГДейки» — бесплатный медиаплан</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>Подготовлено</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="n"/>
+      <c r="P112" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q112" s="2" t="n"/>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>15 лет, 20+ направлений, несколько локаций; мобильный; Zoon ~4 || БАТЧ №10 (FIX plain-text, мультиканальный): отправка чт 17.07; VK/TG-касание D+2</t>
         </is>
       </c>
     </row>
@@ -7680,7 +8380,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4">
@@ -7690,7 +8390,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
@@ -8434,7 +9134,7 @@
         <v>46216</v>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>

</xml_diff>